<commit_message>
docs: update infra to client on-premise server + self-hosted stack
Replace Vercel/Neon/Cloudflare R2/Upstash with:
- Docker + Nginx on client's dedicated server
- Self-hosted PostgreSQL + pgvector
- Self-hosted Redis
- Local disk for file storage
- GitHub (CI/CD) + Sentry free tier only

Monthly infra cost: $0 (client's own server). Updates applied to
ESTIMATE.md, ESTIMATE-3-4-WEEK-DELIVERY.md, and DecisionOS_Estimate.xlsx.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Estimate.xlsx
+++ b/docs/DecisionOS_Estimate.xlsx
@@ -945,7 +945,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>$39–54/month</t>
+          <t>$0/month (client's server)</t>
         </is>
       </c>
     </row>
@@ -1250,22 +1250,22 @@
     <row r="27" ht="19" customHeight="1">
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>Vercel</t>
+          <t>Next.js app</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>Frontend + API Routes + preview deploys</t>
+          <t>Frontend + API Routes (Docker + Nginx)</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Pro</t>
+          <t>Client's server</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>$20</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="F27" s="18" t="inlineStr"/>
@@ -1273,7 +1273,7 @@
     <row r="28" ht="19" customHeight="1">
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>Neon Postgres</t>
+          <t>PostgreSQL + pgvector</t>
         </is>
       </c>
       <c r="C28" s="15" t="inlineStr">
@@ -1283,12 +1283,12 @@
       </c>
       <c r="D28" s="14" t="inlineStr">
         <is>
-          <t>Launch ($19)</t>
+          <t>Self-hosted</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>$19</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="F28" s="15" t="inlineStr"/>
@@ -1296,22 +1296,22 @@
     <row r="29" ht="19" customHeight="1">
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>Cloudflare R2</t>
+          <t>Redis</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>File storage (CSV, Excel, ERP exports)</t>
+          <t>Rate limiting + AI response cache</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Pay-as-you-go</t>
+          <t>Self-hosted</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>$0–5</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="F29" s="18" t="inlineStr"/>
@@ -1319,22 +1319,22 @@
     <row r="30" ht="19" customHeight="1">
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>Upstash Redis</t>
+          <t>Local disk</t>
         </is>
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>Rate limiting + AI response cache</t>
+          <t>File storage — CSV, Excel, ERP exports</t>
         </is>
       </c>
       <c r="D30" s="14" t="inlineStr">
         <is>
-          <t>Pay-as-you-go</t>
+          <t>Client's server</t>
         </is>
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
-          <t>$0–10</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="F30" s="15" t="inlineStr"/>
@@ -1352,7 +1352,7 @@
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Developer</t>
+          <t>Developer (free)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>Source control + CI/CD Actions</t>
+          <t>Source control + CI/CD (SSH deploy)</t>
         </is>
       </c>
       <c r="D32" s="14" t="inlineStr">
@@ -1395,7 +1395,7 @@
       <c r="D33" s="22" t="inlineStr"/>
       <c r="E33" s="16" t="inlineStr">
         <is>
-          <t>$39–54/month</t>
+          <t>$0/month</t>
         </is>
       </c>
       <c r="F33" s="23" t="inlineStr"/>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="G6" s="29" t="inlineStr">
         <is>
-          <t>Drizzle ORM + Neon</t>
+          <t>Drizzle ORM + self-hosted Postgres</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1520,7 @@
       <c r="B7" s="14" t="inlineStr"/>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>Neon/Railway Postgres setup + migrations</t>
+          <t>Self-hosted Postgres setup + pgvector extension + Drizzle migrations</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="G7" s="29" t="inlineStr">
         <is>
-          <t>pgvector extension enabled</t>
+          <t>Runs on client's server</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1699,7 @@
       <c r="B15" s="14" t="inlineStr"/>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>File upload endpoint (multipart → Cloudflare R2 via S3 API)</t>
+          <t>File upload endpoint (multipart → local disk, served via Nginx static path)</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
@@ -2671,7 +2671,7 @@
       <c r="B57" s="14" t="inlineStr"/>
       <c r="C57" s="27" t="inlineStr">
         <is>
-          <t>API rate limiting (Upstash Redis sliding window, per user + per tenant)</t>
+          <t>API rate limiting (self-hosted Redis sliding window, per user + per tenant)</t>
         </is>
       </c>
       <c r="D57" s="14" t="inlineStr">
@@ -2719,7 +2719,7 @@
       <c r="B59" s="14" t="inlineStr"/>
       <c r="C59" s="27" t="inlineStr">
         <is>
-          <t>Query result caching (Upstash Redis, 5-min TTL for repeated AI queries)</t>
+          <t>Query result caching (self-hosted Redis, 5-min TTL for repeated AI queries)</t>
         </is>
       </c>
       <c r="D59" s="14" t="inlineStr">
@@ -2890,7 +2890,7 @@
       <c r="B67" s="14" t="inlineStr"/>
       <c r="C67" s="27" t="inlineStr">
         <is>
-          <t>GitHub Actions CI pipeline (type-check + lint + Vitest + Playwright + Vercel preview)</t>
+          <t>GitHub Actions CI pipeline (type-check + lint + Vitest + Playwright + SSH deploy on merge)</t>
         </is>
       </c>
       <c r="D67" s="14" t="inlineStr">
@@ -2914,7 +2914,7 @@
       <c r="B68" s="14" t="inlineStr"/>
       <c r="C68" s="27" t="inlineStr">
         <is>
-          <t>Production environment setup (Vercel + Neon + Cloudflare R2 + Upstash)</t>
+          <t>Production environment setup (Docker Compose + Nginx + self-hosted Postgres + Redis on client's server)</t>
         </is>
       </c>
       <c r="D68" s="14" t="inlineStr">
@@ -2938,7 +2938,7 @@
       <c r="B69" s="14" t="inlineStr"/>
       <c r="C69" s="27" t="inlineStr">
         <is>
-          <t>Custom domain + SSL + env var management</t>
+          <t>Custom domain + SSL (Let's Encrypt via Certbot + Nginx) + env var management</t>
         </is>
       </c>
       <c r="D69" s="14" t="inlineStr">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="G69" s="29" t="inlineStr">
         <is>
-          <t>Vercel handles SSL automatically</t>
+          <t>Nginx handles SSL termination</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3127,7 @@
           <t>Phase 1: PostgreSQL schema
 (all 7 table groups)
 + Drizzle ORM
-+ Neon setup</t>
++ self-hosted Postgres</t>
         </is>
       </c>
       <c r="D5" s="45" t="inlineStr">
@@ -3148,15 +3148,15 @@
         <is>
           <t>Phase 7: CI/CD pipeline
 (GitHub Actions,
-Vercel, env vars,
-custom domain)</t>
+Docker + SSH deploy,
+Nginx + Let's Encrypt)</t>
         </is>
       </c>
       <c r="G5" s="44" t="inlineStr">
         <is>
           <t>Phase 2: File upload
-+ Cloudflare R2
-storage setup</t>
++ local disk storage
++ Nginx static path</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3279,8 @@
         <is>
           <t>Phase 7: Playwright E2E
 + production deploy
-(Vercel + Neon + R2)</t>
+(Docker + Nginx + Postgres
++ Redis on client server)</t>
         </is>
       </c>
       <c r="G8" s="45" t="inlineStr">
@@ -3327,7 +3328,7 @@
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>Real login + DB on Neon + file upload to R2 + CI/CD pipeline running</t>
+          <t>Real login + self-hosted Postgres live + file upload to local disk + CI/CD pipeline running</t>
         </is>
       </c>
     </row>
@@ -4137,7 +4138,7 @@
       </c>
       <c r="C11" s="27" t="inlineStr">
         <is>
-          <t>Add one CNAME record to point your domain to Vercel. We will provide the value.</t>
+          <t>Point your domain's A record to the client server's IP address. We will provide the IP once the server is set up.</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -4166,7 +4167,7 @@
       </c>
       <c r="C13" s="27" t="inlineStr">
         <is>
-          <t>How many tenant organisations at go-live? Informs connection pool sizing on Neon and initial seed data needed.</t>
+          <t>How many tenant organisations at go-live? Informs connection pool sizing on the self-hosted Postgres instance.</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">

</xml_diff>

<commit_message>
docs: remove Google Sheets and Salesforce connectors from estimate
Both connectors removed from Phase 3, third-party connector costs table,
MVP cuts list, and post-launch sections across all three estimate files.
Phase 3 total unchanged at 13 days (these were already labelled post-launch
and excluded from the billing total).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Estimate.xlsx
+++ b/docs/DecisionOS_Estimate.xlsx
@@ -1159,7 +1159,7 @@
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>Data Connectors (Zoho + Custom ERP + PgSQL)</t>
+          <t>Data Connectors (Zoho CRM + Custom ERP + PostgreSQL direct)</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
@@ -1604,7 +1604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I72"/>
+  <dimension ref="B1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2389,147 +2389,135 @@
       <c r="I27" s="34" t="inlineStr"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="B28" s="14" t="inlineStr"/>
-      <c r="C28" s="31" t="inlineStr">
-        <is>
-          <t>Google Sheets connector (OAuth + Sheets API v4)</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Phase 3 Total</t>
+        </is>
+      </c>
+      <c r="C28" s="35" t="inlineStr"/>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>13 days</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>104 hrs</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>$2,080</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>28 days</t>
+        </is>
+      </c>
+      <c r="H28" s="36" t="inlineStr"/>
+      <c r="I28" s="37" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Phase 4  —  AI / LLM Engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="B30" s="14" t="inlineStr"/>
+      <c r="C30" s="31" t="inlineStr">
+        <is>
+          <t>pgvector extension + embedding schema</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>0.5 day</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>4 hrs</t>
+        </is>
+      </c>
+      <c r="F30" s="16" t="inlineStr">
+        <is>
+          <t>$80</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
         <is>
           <t>2 days</t>
         </is>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="H30" s="32" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="I30" s="34" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="B31" s="14" t="inlineStr"/>
+      <c r="C31" s="31" t="inlineStr">
+        <is>
+          <t>Embedding pipeline — chunk rows → embed via provider → store vectors</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>2 days</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
         <is>
           <t>16 hrs</t>
         </is>
       </c>
-      <c r="F28" s="16" t="inlineStr">
+      <c r="F31" s="16" t="inlineStr">
         <is>
           <t>$320</t>
         </is>
       </c>
-      <c r="G28" s="14" t="inlineStr">
-        <is>
-          <t>4 days</t>
-        </is>
-      </c>
-      <c r="H28" s="39" t="inlineStr">
-        <is>
-          <t>Post-launch</t>
-        </is>
-      </c>
-      <c r="I28" s="33" t="inlineStr">
-        <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="B29" s="14" t="inlineStr"/>
-      <c r="C29" s="31" t="inlineStr">
-        <is>
-          <t>Salesforce connector (OAuth 2.0 PKCE + SOQL)</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="inlineStr">
-        <is>
-          <t>3 days</t>
-        </is>
-      </c>
-      <c r="E29" s="14" t="inlineStr">
-        <is>
-          <t>24 hrs</t>
-        </is>
-      </c>
-      <c r="F29" s="16" t="inlineStr">
-        <is>
-          <t>$480</t>
-        </is>
-      </c>
-      <c r="G29" s="14" t="inlineStr">
-        <is>
-          <t>7 days</t>
-        </is>
-      </c>
-      <c r="H29" s="39" t="inlineStr">
-        <is>
-          <t>Post-launch</t>
-        </is>
-      </c>
-      <c r="I29" s="33" t="inlineStr">
-        <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>Phase 3 Total (Launch)</t>
-        </is>
-      </c>
-      <c r="C30" s="35" t="inlineStr"/>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>13 days</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>104 hrs</t>
-        </is>
-      </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>$2,080</t>
-        </is>
-      </c>
-      <c r="G30" s="8" t="inlineStr">
-        <is>
-          <t>28 days</t>
-        </is>
-      </c>
-      <c r="H30" s="36" t="inlineStr"/>
-      <c r="I30" s="33" t="inlineStr">
-        <is>
-          <t>Post-launch: +5 days</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="B31" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Phase 4  —  AI / LLM Engine</t>
-        </is>
-      </c>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>5 days</t>
+        </is>
+      </c>
+      <c r="H31" s="32" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="I31" s="34" t="inlineStr"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="B32" s="14" t="inlineStr"/>
       <c r="C32" s="31" t="inlineStr">
         <is>
-          <t>pgvector extension + embedding schema</t>
+          <t>RAG retrieval — query → embed → cosine similarity → context assembly</t>
         </is>
       </c>
       <c r="D32" s="14" t="inlineStr">
         <is>
-          <t>0.5 day</t>
+          <t>2 days</t>
         </is>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>4 hrs</t>
+          <t>16 hrs</t>
         </is>
       </c>
       <c r="F32" s="16" t="inlineStr">
         <is>
-          <t>$80</t>
+          <t>$320</t>
         </is>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>6 days</t>
         </is>
       </c>
       <c r="H32" s="32" t="inlineStr">
@@ -2543,7 +2531,7 @@
       <c r="B33" s="14" t="inlineStr"/>
       <c r="C33" s="31" t="inlineStr">
         <is>
-          <t>Embedding pipeline — chunk rows → embed via provider → store vectors</t>
+          <t>SQL generation — LLM → SQL → AST safety check (SELECT-only) → execute → citations</t>
         </is>
       </c>
       <c r="D33" s="14" t="inlineStr">
@@ -2571,13 +2559,17 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="I33" s="34" t="inlineStr"/>
+      <c r="I33" s="33" t="inlineStr">
+        <is>
+          <t>node-sql-parser prevents writes</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="B34" s="14" t="inlineStr"/>
       <c r="C34" s="31" t="inlineStr">
         <is>
-          <t>RAG retrieval — query → embed → cosine similarity → context assembly</t>
+          <t>Multi-provider LLM router — routes to tenant's configured provider</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -2597,7 +2589,7 @@
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
-          <t>6 days</t>
+          <t>4 days</t>
         </is>
       </c>
       <c r="H34" s="32" t="inlineStr">
@@ -2611,7 +2603,7 @@
       <c r="B35" s="14" t="inlineStr"/>
       <c r="C35" s="31" t="inlineStr">
         <is>
-          <t>SQL generation — LLM → SQL → AST safety check (SELECT-only) → execute → citations</t>
+          <t>LLM provider integrations: Anthropic Claude, OpenAI GPT-4o, Google Gemini</t>
         </is>
       </c>
       <c r="D35" s="14" t="inlineStr">
@@ -2641,7 +2633,7 @@
       </c>
       <c r="I35" s="33" t="inlineStr">
         <is>
-          <t>node-sql-parser prevents writes</t>
+          <t>Tenant supplies own API keys</t>
         </is>
       </c>
     </row>
@@ -2649,71 +2641,75 @@
       <c r="B36" s="14" t="inlineStr"/>
       <c r="C36" s="31" t="inlineStr">
         <is>
-          <t>Multi-provider LLM router — routes to tenant's configured provider</t>
+          <t>LLM Connect wizard — provider selector → paste API key → test connection → save default</t>
         </is>
       </c>
       <c r="D36" s="14" t="inlineStr">
         <is>
+          <t>1 day</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="inlineStr">
+        <is>
+          <t>8 hrs</t>
+        </is>
+      </c>
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>$160</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="inlineStr">
+        <is>
           <t>2 days</t>
         </is>
       </c>
-      <c r="E36" s="14" t="inlineStr">
-        <is>
-          <t>16 hrs</t>
-        </is>
-      </c>
-      <c r="F36" s="16" t="inlineStr">
-        <is>
-          <t>$320</t>
-        </is>
-      </c>
-      <c r="G36" s="14" t="inlineStr">
-        <is>
-          <t>4 days</t>
-        </is>
-      </c>
-      <c r="H36" s="32" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="I36" s="34" t="inlineStr"/>
+      <c r="H36" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I36" s="33" t="inlineStr">
+        <is>
+          <t>Simple wizard-style UX</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="B37" s="14" t="inlineStr"/>
       <c r="C37" s="31" t="inlineStr">
         <is>
-          <t>LLM provider integrations: Anthropic Claude, OpenAI GPT-4o, Google Gemini</t>
+          <t>LLM usage logging — llm_usage_logs table (tokens, cost_estimate, provider, user)</t>
         </is>
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>0.5 day</t>
         </is>
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
-          <t>16 hrs</t>
+          <t>4 hrs</t>
         </is>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
-          <t>$320</t>
+          <t>$80</t>
         </is>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
-          <t>5 days</t>
-        </is>
-      </c>
-      <c r="H37" s="32" t="inlineStr">
-        <is>
-          <t>Critical</t>
+          <t>1 day</t>
+        </is>
+      </c>
+      <c r="H37" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="I37" s="33" t="inlineStr">
         <is>
-          <t>Tenant supplies own API keys</t>
+          <t>Foundation for usage dashboard</t>
         </is>
       </c>
     </row>
@@ -2721,37 +2717,37 @@
       <c r="B38" s="14" t="inlineStr"/>
       <c r="C38" s="31" t="inlineStr">
         <is>
-          <t>LLM Connect wizard — provider selector → paste API key → test connection → save default</t>
+          <t>7-agent orchestration — Intent → Governance (PII masking) → Data Analyst → BI → Insight → Recommendation → Workflow</t>
         </is>
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
-          <t>1 day</t>
+          <t>4 days</t>
         </is>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
-          <t>8 hrs</t>
+          <t>32 hrs</t>
         </is>
       </c>
       <c r="F38" s="16" t="inlineStr">
         <is>
-          <t>$160</t>
+          <t>$640</t>
         </is>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
-          <t>2 days</t>
-        </is>
-      </c>
-      <c r="H38" s="38" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>9 days</t>
+        </is>
+      </c>
+      <c r="H38" s="32" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I38" s="33" t="inlineStr">
         <is>
-          <t>Simple wizard-style UX</t>
+          <t>Strong model for analyst/insight/rec; fast for others</t>
         </is>
       </c>
     </row>
@@ -2759,37 +2755,37 @@
       <c r="B39" s="14" t="inlineStr"/>
       <c r="C39" s="31" t="inlineStr">
         <is>
-          <t>LLM usage logging — llm_usage_logs table (tokens, cost_estimate, provider, user)</t>
+          <t>Chat session persistence — chat_sessions + chat_messages CRUD API, session list, pagination</t>
         </is>
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>0.5 day</t>
+          <t>1 day</t>
         </is>
       </c>
       <c r="E39" s="14" t="inlineStr">
         <is>
-          <t>4 hrs</t>
+          <t>8 hrs</t>
         </is>
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
-          <t>$80</t>
+          <t>$160</t>
         </is>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
-          <t>1 day</t>
-        </is>
-      </c>
-      <c r="H39" s="38" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>2 days</t>
+        </is>
+      </c>
+      <c r="H39" s="32" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I39" s="33" t="inlineStr">
         <is>
-          <t>Foundation for usage dashboard</t>
+          <t>Feeds session sidebar</t>
         </is>
       </c>
     </row>
@@ -2797,27 +2793,27 @@
       <c r="B40" s="14" t="inlineStr"/>
       <c r="C40" s="31" t="inlineStr">
         <is>
-          <t>7-agent orchestration — Intent → Governance (PII masking) → Data Analyst → BI → Insight → Recommendation → Workflow</t>
+          <t>SSE streaming — AI response streams token-by-token to chat UI</t>
         </is>
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>4 days</t>
+          <t>1 day</t>
         </is>
       </c>
       <c r="E40" s="14" t="inlineStr">
         <is>
-          <t>32 hrs</t>
+          <t>8 hrs</t>
         </is>
       </c>
       <c r="F40" s="16" t="inlineStr">
         <is>
-          <t>$640</t>
+          <t>$160</t>
         </is>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
-          <t>9 days</t>
+          <t>2 days</t>
         </is>
       </c>
       <c r="H40" s="32" t="inlineStr">
@@ -2825,17 +2821,13 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="I40" s="33" t="inlineStr">
-        <is>
-          <t>Strong model for analyst/insight/rec; fast for others</t>
-        </is>
-      </c>
+      <c r="I40" s="34" t="inlineStr"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="B41" s="14" t="inlineStr"/>
       <c r="C41" s="31" t="inlineStr">
         <is>
-          <t>Chat session persistence — chat_sessions + chat_messages CRUD API, session list, pagination</t>
+          <t>AI Executive Summary generator — nightly cron per tenant</t>
         </is>
       </c>
       <c r="D41" s="14" t="inlineStr">
@@ -2855,189 +2847,185 @@
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
-          <t>2 days</t>
-        </is>
-      </c>
-      <c r="H41" s="32" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="I41" s="33" t="inlineStr">
-        <is>
-          <t>Feeds session sidebar</t>
-        </is>
-      </c>
+          <t>3 days</t>
+        </is>
+      </c>
+      <c r="H41" s="39" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I41" s="34" t="inlineStr"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="14" t="inlineStr"/>
       <c r="C42" s="31" t="inlineStr">
         <is>
-          <t>SSE streaming — AI response streams token-by-token to chat UI</t>
+          <t>Insight + Recommendation auto-generation (LLM + threshold rule engine, 4h cron)</t>
         </is>
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>1 day</t>
+          <t>2 days</t>
         </is>
       </c>
       <c r="E42" s="14" t="inlineStr">
         <is>
-          <t>8 hrs</t>
+          <t>16 hrs</t>
         </is>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
-          <t>$160</t>
+          <t>$320</t>
         </is>
       </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
+          <t>5 days</t>
+        </is>
+      </c>
+      <c r="H42" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I42" s="34" t="inlineStr"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>Phase 4 Total</t>
+        </is>
+      </c>
+      <c r="C43" s="35" t="inlineStr"/>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>21 days</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>168 hrs</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>$3,360</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>51 days</t>
+        </is>
+      </c>
+      <c r="H43" s="36" t="inlineStr"/>
+      <c r="I43" s="37" t="inlineStr"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="B44" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Phase 5  —  Frontend Integration + Subscription Enforcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="B45" s="14" t="inlineStr"/>
+      <c r="C45" s="31" t="inlineStr">
+        <is>
+          <t>TanStack Query hooks for all endpoints (users, KPIs, insights, recommendations, tasks)</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr">
+        <is>
           <t>2 days</t>
         </is>
       </c>
-      <c r="H42" s="32" t="inlineStr">
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>16 hrs</t>
+        </is>
+      </c>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
+          <t>$320</t>
+        </is>
+      </c>
+      <c r="G45" s="14" t="inlineStr">
+        <is>
+          <t>4 days</t>
+        </is>
+      </c>
+      <c r="H45" s="32" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I42" s="34" t="inlineStr"/>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="B43" s="14" t="inlineStr"/>
-      <c r="C43" s="31" t="inlineStr">
-        <is>
-          <t>AI Executive Summary generator — nightly cron per tenant</t>
-        </is>
-      </c>
-      <c r="D43" s="14" t="inlineStr">
-        <is>
-          <t>1 day</t>
-        </is>
-      </c>
-      <c r="E43" s="14" t="inlineStr">
-        <is>
-          <t>8 hrs</t>
-        </is>
-      </c>
-      <c r="F43" s="16" t="inlineStr">
-        <is>
-          <t>$160</t>
-        </is>
-      </c>
-      <c r="G43" s="14" t="inlineStr">
-        <is>
-          <t>3 days</t>
-        </is>
-      </c>
-      <c r="H43" s="39" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I43" s="34" t="inlineStr"/>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="B44" s="14" t="inlineStr"/>
-      <c r="C44" s="31" t="inlineStr">
-        <is>
-          <t>Insight + Recommendation auto-generation (LLM + threshold rule engine, 4h cron)</t>
-        </is>
-      </c>
-      <c r="D44" s="14" t="inlineStr">
+      <c r="I45" s="34" t="inlineStr"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="B46" s="14" t="inlineStr"/>
+      <c r="C46" s="31" t="inlineStr">
+        <is>
+          <t>Real KPI computation (SQL aggregates per tenant, configurable formulas)</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="inlineStr">
         <is>
           <t>2 days</t>
         </is>
       </c>
-      <c r="E44" s="14" t="inlineStr">
+      <c r="E46" s="14" t="inlineStr">
         <is>
           <t>16 hrs</t>
         </is>
       </c>
-      <c r="F44" s="16" t="inlineStr">
+      <c r="F46" s="16" t="inlineStr">
         <is>
           <t>$320</t>
         </is>
       </c>
-      <c r="G44" s="14" t="inlineStr">
-        <is>
-          <t>5 days</t>
-        </is>
-      </c>
-      <c r="H44" s="38" t="inlineStr">
+      <c r="G46" s="14" t="inlineStr">
+        <is>
+          <t>4 days</t>
+        </is>
+      </c>
+      <c r="H46" s="38" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I44" s="34" t="inlineStr"/>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t>Phase 4 Total</t>
-        </is>
-      </c>
-      <c r="C45" s="35" t="inlineStr"/>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>21 days</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>168 hrs</t>
-        </is>
-      </c>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>$3,360</t>
-        </is>
-      </c>
-      <c r="G45" s="8" t="inlineStr">
-        <is>
-          <t>51 days</t>
-        </is>
-      </c>
-      <c r="H45" s="36" t="inlineStr"/>
-      <c r="I45" s="37" t="inlineStr"/>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="B46" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Phase 5  —  Frontend Integration + Subscription Enforcement</t>
-        </is>
-      </c>
+      <c r="I46" s="34" t="inlineStr"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="B47" s="14" t="inlineStr"/>
       <c r="C47" s="31" t="inlineStr">
         <is>
-          <t>TanStack Query hooks for all endpoints (users, KPIs, insights, recommendations, tasks)</t>
+          <t>Real dashboard charts (live data → Recharts via API)</t>
         </is>
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
+          <t>1 day</t>
+        </is>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>8 hrs</t>
+        </is>
+      </c>
+      <c r="F47" s="16" t="inlineStr">
+        <is>
+          <t>$160</t>
+        </is>
+      </c>
+      <c r="G47" s="14" t="inlineStr">
+        <is>
           <t>2 days</t>
         </is>
       </c>
-      <c r="E47" s="14" t="inlineStr">
-        <is>
-          <t>16 hrs</t>
-        </is>
-      </c>
-      <c r="F47" s="16" t="inlineStr">
-        <is>
-          <t>$320</t>
-        </is>
-      </c>
-      <c r="G47" s="14" t="inlineStr">
-        <is>
-          <t>4 days</t>
-        </is>
-      </c>
-      <c r="H47" s="32" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="H47" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="I47" s="34" t="inlineStr"/>
@@ -3046,32 +3034,32 @@
       <c r="B48" s="14" t="inlineStr"/>
       <c r="C48" s="31" t="inlineStr">
         <is>
-          <t>Real KPI computation (SQL aggregates per tenant, configurable formulas)</t>
+          <t>Notification system (SSE endpoint → existing notification bell)</t>
         </is>
       </c>
       <c r="D48" s="14" t="inlineStr">
         <is>
+          <t>1 day</t>
+        </is>
+      </c>
+      <c r="E48" s="14" t="inlineStr">
+        <is>
+          <t>8 hrs</t>
+        </is>
+      </c>
+      <c r="F48" s="16" t="inlineStr">
+        <is>
+          <t>$160</t>
+        </is>
+      </c>
+      <c r="G48" s="14" t="inlineStr">
+        <is>
           <t>2 days</t>
         </is>
       </c>
-      <c r="E48" s="14" t="inlineStr">
-        <is>
-          <t>16 hrs</t>
-        </is>
-      </c>
-      <c r="F48" s="16" t="inlineStr">
-        <is>
-          <t>$320</t>
-        </is>
-      </c>
-      <c r="G48" s="14" t="inlineStr">
-        <is>
-          <t>4 days</t>
-        </is>
-      </c>
-      <c r="H48" s="38" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="H48" s="39" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I48" s="34" t="inlineStr"/>
@@ -3080,7 +3068,7 @@
       <c r="B49" s="14" t="inlineStr"/>
       <c r="C49" s="31" t="inlineStr">
         <is>
-          <t>Real dashboard charts (live data → Recharts via API)</t>
+          <t>Workflow / task CRUD persistence</t>
         </is>
       </c>
       <c r="D49" s="14" t="inlineStr">
@@ -3103,9 +3091,9 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H49" s="38" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="H49" s="39" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I49" s="34" t="inlineStr"/>
@@ -3114,7 +3102,7 @@
       <c r="B50" s="14" t="inlineStr"/>
       <c r="C50" s="31" t="inlineStr">
         <is>
-          <t>Notification system (SSE endpoint → existing notification bell)</t>
+          <t>Subscription enforcement middleware — user + data source limits → 402 on breach</t>
         </is>
       </c>
       <c r="D50" s="14" t="inlineStr">
@@ -3134,21 +3122,25 @@
       </c>
       <c r="G50" s="14" t="inlineStr">
         <is>
-          <t>2 days</t>
-        </is>
-      </c>
-      <c r="H50" s="39" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I50" s="34" t="inlineStr"/>
+          <t>3 days</t>
+        </is>
+      </c>
+      <c r="H50" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I50" s="33" t="inlineStr">
+        <is>
+          <t>No query cap — tenant pays own LLM</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="B51" s="14" t="inlineStr"/>
       <c r="C51" s="31" t="inlineStr">
         <is>
-          <t>Workflow / task CRUD persistence</t>
+          <t>Tenant Admin Console — LLM wizard + usage dashboard (tokens, cost estimate, per-user)</t>
         </is>
       </c>
       <c r="D51" s="14" t="inlineStr">
@@ -3171,9 +3163,9 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H51" s="39" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="H51" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="I51" s="34" t="inlineStr"/>
@@ -3182,150 +3174,146 @@
       <c r="B52" s="14" t="inlineStr"/>
       <c r="C52" s="31" t="inlineStr">
         <is>
-          <t>Subscription enforcement middleware — user + data source limits → 402 on breach</t>
+          <t>Platform Admin panel — plan CRUD, per-tenant plan assignment</t>
         </is>
       </c>
       <c r="D52" s="14" t="inlineStr">
         <is>
+          <t>0.5 day</t>
+        </is>
+      </c>
+      <c r="E52" s="14" t="inlineStr">
+        <is>
+          <t>4 hrs</t>
+        </is>
+      </c>
+      <c r="F52" s="16" t="inlineStr">
+        <is>
+          <t>$80</t>
+        </is>
+      </c>
+      <c r="G52" s="14" t="inlineStr">
+        <is>
           <t>1 day</t>
         </is>
       </c>
-      <c r="E52" s="14" t="inlineStr">
+      <c r="H52" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I52" s="34" t="inlineStr"/>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>Phase 5 Total</t>
+        </is>
+      </c>
+      <c r="C53" s="35" t="inlineStr"/>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>9.5 days</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>76 hrs</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>$1,520</t>
+        </is>
+      </c>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>20 days</t>
+        </is>
+      </c>
+      <c r="H53" s="36" t="inlineStr"/>
+      <c r="I53" s="37" t="inlineStr"/>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="B54" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Phase 6  —  Production Hardening</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="B55" s="14" t="inlineStr"/>
+      <c r="C55" s="31" t="inlineStr">
+        <is>
+          <t>API rate limiting (self-hosted Redis sliding window, per user + per tenant)</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>1 day</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr">
         <is>
           <t>8 hrs</t>
         </is>
       </c>
-      <c r="F52" s="16" t="inlineStr">
+      <c r="F55" s="16" t="inlineStr">
         <is>
           <t>$160</t>
         </is>
       </c>
-      <c r="G52" s="14" t="inlineStr">
-        <is>
-          <t>3 days</t>
-        </is>
-      </c>
-      <c r="H52" s="38" t="inlineStr">
+      <c r="G55" s="14" t="inlineStr">
+        <is>
+          <t>2 days</t>
+        </is>
+      </c>
+      <c r="H55" s="38" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I52" s="33" t="inlineStr">
-        <is>
-          <t>No query cap — tenant pays own LLM</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="B53" s="14" t="inlineStr"/>
-      <c r="C53" s="31" t="inlineStr">
-        <is>
-          <t>Tenant Admin Console — LLM wizard + usage dashboard (tokens, cost estimate, per-user)</t>
-        </is>
-      </c>
-      <c r="D53" s="14" t="inlineStr">
+      <c r="I55" s="34" t="inlineStr"/>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="B56" s="14" t="inlineStr"/>
+      <c r="C56" s="31" t="inlineStr">
+        <is>
+          <t>Error boundaries + structured logging (Sentry + Pino)</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
         <is>
           <t>1 day</t>
         </is>
       </c>
-      <c r="E53" s="14" t="inlineStr">
+      <c r="E56" s="14" t="inlineStr">
         <is>
           <t>8 hrs</t>
         </is>
       </c>
-      <c r="F53" s="16" t="inlineStr">
+      <c r="F56" s="16" t="inlineStr">
         <is>
           <t>$160</t>
         </is>
       </c>
-      <c r="G53" s="14" t="inlineStr">
+      <c r="G56" s="14" t="inlineStr">
         <is>
           <t>2 days</t>
         </is>
       </c>
-      <c r="H53" s="38" t="inlineStr">
+      <c r="H56" s="38" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I53" s="34" t="inlineStr"/>
-    </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="B54" s="14" t="inlineStr"/>
-      <c r="C54" s="31" t="inlineStr">
-        <is>
-          <t>Platform Admin panel — plan CRUD, per-tenant plan assignment</t>
-        </is>
-      </c>
-      <c r="D54" s="14" t="inlineStr">
-        <is>
-          <t>0.5 day</t>
-        </is>
-      </c>
-      <c r="E54" s="14" t="inlineStr">
-        <is>
-          <t>4 hrs</t>
-        </is>
-      </c>
-      <c r="F54" s="16" t="inlineStr">
-        <is>
-          <t>$80</t>
-        </is>
-      </c>
-      <c r="G54" s="14" t="inlineStr">
-        <is>
-          <t>1 day</t>
-        </is>
-      </c>
-      <c r="H54" s="38" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I54" s="34" t="inlineStr"/>
-    </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>Phase 5 Total</t>
-        </is>
-      </c>
-      <c r="C55" s="35" t="inlineStr"/>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>9.5 days</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>76 hrs</t>
-        </is>
-      </c>
-      <c r="F55" s="8" t="inlineStr">
-        <is>
-          <t>$1,520</t>
-        </is>
-      </c>
-      <c r="G55" s="8" t="inlineStr">
-        <is>
-          <t>20 days</t>
-        </is>
-      </c>
-      <c r="H55" s="36" t="inlineStr"/>
-      <c r="I55" s="37" t="inlineStr"/>
-    </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="B56" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Phase 6  —  Production Hardening</t>
-        </is>
-      </c>
+      <c r="I56" s="34" t="inlineStr"/>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="B57" s="14" t="inlineStr"/>
       <c r="C57" s="31" t="inlineStr">
         <is>
-          <t>API rate limiting (self-hosted Redis sliding window, per user + per tenant)</t>
+          <t>Query result caching (self-hosted Redis, 5-min TTL for repeated AI queries)</t>
         </is>
       </c>
       <c r="D57" s="14" t="inlineStr">
@@ -3345,12 +3333,12 @@
       </c>
       <c r="G57" s="14" t="inlineStr">
         <is>
-          <t>2 days</t>
-        </is>
-      </c>
-      <c r="H57" s="38" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>3 days</t>
+        </is>
+      </c>
+      <c r="H57" s="39" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I57" s="34" t="inlineStr"/>
@@ -3359,7 +3347,7 @@
       <c r="B58" s="14" t="inlineStr"/>
       <c r="C58" s="31" t="inlineStr">
         <is>
-          <t>Error boundaries + structured logging (Sentry + Pino)</t>
+          <t>Security audit — SQL injection, XSS, OWASP headers, CSRF</t>
         </is>
       </c>
       <c r="D58" s="14" t="inlineStr">
@@ -3379,7 +3367,7 @@
       </c>
       <c r="G58" s="14" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>3 days</t>
         </is>
       </c>
       <c r="H58" s="38" t="inlineStr">
@@ -3393,22 +3381,22 @@
       <c r="B59" s="14" t="inlineStr"/>
       <c r="C59" s="31" t="inlineStr">
         <is>
-          <t>Query result caching (self-hosted Redis, 5-min TTL for repeated AI queries)</t>
+          <t>Multi-tenant data isolation audit — cross-tenant pen-test</t>
         </is>
       </c>
       <c r="D59" s="14" t="inlineStr">
         <is>
-          <t>1 day</t>
+          <t>0.5 day</t>
         </is>
       </c>
       <c r="E59" s="14" t="inlineStr">
         <is>
-          <t>8 hrs</t>
+          <t>4 hrs</t>
         </is>
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>$160</t>
+          <t>$80</t>
         </is>
       </c>
       <c r="G59" s="14" t="inlineStr">
@@ -3416,9 +3404,9 @@
           <t>3 days</t>
         </is>
       </c>
-      <c r="H59" s="39" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="H59" s="32" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I59" s="34" t="inlineStr"/>
@@ -3427,29 +3415,29 @@
       <c r="B60" s="14" t="inlineStr"/>
       <c r="C60" s="31" t="inlineStr">
         <is>
-          <t>Security audit — SQL injection, XSS, OWASP headers, CSRF</t>
+          <t>Password policy + account lockout</t>
         </is>
       </c>
       <c r="D60" s="14" t="inlineStr">
         <is>
+          <t>0.5 day</t>
+        </is>
+      </c>
+      <c r="E60" s="14" t="inlineStr">
+        <is>
+          <t>4 hrs</t>
+        </is>
+      </c>
+      <c r="F60" s="16" t="inlineStr">
+        <is>
+          <t>$80</t>
+        </is>
+      </c>
+      <c r="G60" s="14" t="inlineStr">
+        <is>
           <t>1 day</t>
         </is>
       </c>
-      <c r="E60" s="14" t="inlineStr">
-        <is>
-          <t>8 hrs</t>
-        </is>
-      </c>
-      <c r="F60" s="16" t="inlineStr">
-        <is>
-          <t>$160</t>
-        </is>
-      </c>
-      <c r="G60" s="14" t="inlineStr">
-        <is>
-          <t>3 days</t>
-        </is>
-      </c>
       <c r="H60" s="38" t="inlineStr">
         <is>
           <t>High</t>
@@ -3458,135 +3446,135 @@
       <c r="I60" s="34" t="inlineStr"/>
     </row>
     <row r="61" ht="20" customHeight="1">
-      <c r="B61" s="14" t="inlineStr"/>
-      <c r="C61" s="31" t="inlineStr">
-        <is>
-          <t>Multi-tenant data isolation audit — cross-tenant pen-test</t>
-        </is>
-      </c>
-      <c r="D61" s="14" t="inlineStr">
-        <is>
-          <t>0.5 day</t>
-        </is>
-      </c>
-      <c r="E61" s="14" t="inlineStr">
-        <is>
-          <t>4 hrs</t>
-        </is>
-      </c>
-      <c r="F61" s="16" t="inlineStr">
-        <is>
-          <t>$80</t>
-        </is>
-      </c>
-      <c r="G61" s="14" t="inlineStr">
-        <is>
-          <t>3 days</t>
-        </is>
-      </c>
-      <c r="H61" s="32" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="I61" s="34" t="inlineStr"/>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>Phase 6 Total</t>
+        </is>
+      </c>
+      <c r="C61" s="35" t="inlineStr"/>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>5 days</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>40 hrs</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="inlineStr">
+        <is>
+          <t>$800</t>
+        </is>
+      </c>
+      <c r="G61" s="8" t="inlineStr">
+        <is>
+          <t>14 days</t>
+        </is>
+      </c>
+      <c r="H61" s="36" t="inlineStr"/>
+      <c r="I61" s="37" t="inlineStr"/>
     </row>
     <row r="62" ht="20" customHeight="1">
-      <c r="B62" s="14" t="inlineStr"/>
-      <c r="C62" s="31" t="inlineStr">
-        <is>
-          <t>Password policy + account lockout</t>
-        </is>
-      </c>
-      <c r="D62" s="14" t="inlineStr">
-        <is>
-          <t>0.5 day</t>
-        </is>
-      </c>
-      <c r="E62" s="14" t="inlineStr">
-        <is>
-          <t>4 hrs</t>
-        </is>
-      </c>
-      <c r="F62" s="16" t="inlineStr">
-        <is>
-          <t>$80</t>
-        </is>
-      </c>
-      <c r="G62" s="14" t="inlineStr">
-        <is>
-          <t>1 day</t>
-        </is>
-      </c>
-      <c r="H62" s="38" t="inlineStr">
+      <c r="B62" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Phase 7  —  QA, CI/CD &amp; Deployment</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="B63" s="14" t="inlineStr"/>
+      <c r="C63" s="31" t="inlineStr">
+        <is>
+          <t>Unit + integration tests (Vitest — API routes, auth, data ingestion, LLM router)</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>2 days</t>
+        </is>
+      </c>
+      <c r="E63" s="14" t="inlineStr">
+        <is>
+          <t>16 hrs</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="inlineStr">
+        <is>
+          <t>$320</t>
+        </is>
+      </c>
+      <c r="G63" s="14" t="inlineStr">
+        <is>
+          <t>5 days</t>
+        </is>
+      </c>
+      <c r="H63" s="38" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I62" s="34" t="inlineStr"/>
-    </row>
-    <row r="63" ht="20" customHeight="1">
-      <c r="B63" s="8" t="inlineStr">
-        <is>
-          <t>Phase 6 Total</t>
-        </is>
-      </c>
-      <c r="C63" s="35" t="inlineStr"/>
-      <c r="D63" s="8" t="inlineStr">
+      <c r="I63" s="34" t="inlineStr"/>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="B64" s="14" t="inlineStr"/>
+      <c r="C64" s="31" t="inlineStr">
+        <is>
+          <t>E2E tests (Playwright — login, upload CSV, Zoho connect, ask AI, workflow create)</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>2 days</t>
+        </is>
+      </c>
+      <c r="E64" s="14" t="inlineStr">
+        <is>
+          <t>16 hrs</t>
+        </is>
+      </c>
+      <c r="F64" s="16" t="inlineStr">
+        <is>
+          <t>$320</t>
+        </is>
+      </c>
+      <c r="G64" s="14" t="inlineStr">
         <is>
           <t>5 days</t>
         </is>
       </c>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>40 hrs</t>
-        </is>
-      </c>
-      <c r="F63" s="8" t="inlineStr">
-        <is>
-          <t>$800</t>
-        </is>
-      </c>
-      <c r="G63" s="8" t="inlineStr">
-        <is>
-          <t>14 days</t>
-        </is>
-      </c>
-      <c r="H63" s="36" t="inlineStr"/>
-      <c r="I63" s="37" t="inlineStr"/>
-    </row>
-    <row r="64" ht="20" customHeight="1">
-      <c r="B64" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Phase 7  —  QA, CI/CD &amp; Deployment</t>
-        </is>
-      </c>
+      <c r="H64" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I64" s="34" t="inlineStr"/>
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="B65" s="14" t="inlineStr"/>
       <c r="C65" s="31" t="inlineStr">
         <is>
-          <t>Unit + integration tests (Vitest — API routes, auth, data ingestion, LLM router)</t>
+          <t>GitHub Actions CI pipeline (type-check + lint + Vitest + Playwright + SSH deploy on merge)</t>
         </is>
       </c>
       <c r="D65" s="14" t="inlineStr">
         <is>
+          <t>1 day</t>
+        </is>
+      </c>
+      <c r="E65" s="14" t="inlineStr">
+        <is>
+          <t>8 hrs</t>
+        </is>
+      </c>
+      <c r="F65" s="16" t="inlineStr">
+        <is>
+          <t>$160</t>
+        </is>
+      </c>
+      <c r="G65" s="14" t="inlineStr">
+        <is>
           <t>2 days</t>
-        </is>
-      </c>
-      <c r="E65" s="14" t="inlineStr">
-        <is>
-          <t>16 hrs</t>
-        </is>
-      </c>
-      <c r="F65" s="16" t="inlineStr">
-        <is>
-          <t>$320</t>
-        </is>
-      </c>
-      <c r="G65" s="14" t="inlineStr">
-        <is>
-          <t>5 days</t>
         </is>
       </c>
       <c r="H65" s="38" t="inlineStr">
@@ -3600,32 +3588,32 @@
       <c r="B66" s="14" t="inlineStr"/>
       <c r="C66" s="31" t="inlineStr">
         <is>
-          <t>E2E tests (Playwright — login, upload CSV, Zoho connect, ask AI, workflow create)</t>
+          <t>Production environment setup (Docker Compose + Nginx + self-hosted Postgres + Redis on client's server)</t>
         </is>
       </c>
       <c r="D66" s="14" t="inlineStr">
         <is>
-          <t>2 days</t>
+          <t>0.5 day</t>
         </is>
       </c>
       <c r="E66" s="14" t="inlineStr">
         <is>
-          <t>16 hrs</t>
+          <t>4 hrs</t>
         </is>
       </c>
       <c r="F66" s="16" t="inlineStr">
         <is>
-          <t>$320</t>
+          <t>$80</t>
         </is>
       </c>
       <c r="G66" s="14" t="inlineStr">
         <is>
-          <t>5 days</t>
-        </is>
-      </c>
-      <c r="H66" s="38" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>1 day</t>
+        </is>
+      </c>
+      <c r="H66" s="32" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I66" s="34" t="inlineStr"/>
@@ -3634,41 +3622,45 @@
       <c r="B67" s="14" t="inlineStr"/>
       <c r="C67" s="31" t="inlineStr">
         <is>
-          <t>GitHub Actions CI pipeline (type-check + lint + Vitest + Playwright + SSH deploy on merge)</t>
+          <t>Custom domain + SSL (Let's Encrypt via Certbot + Nginx) + env var management</t>
         </is>
       </c>
       <c r="D67" s="14" t="inlineStr">
         <is>
+          <t>0.5 day</t>
+        </is>
+      </c>
+      <c r="E67" s="14" t="inlineStr">
+        <is>
+          <t>4 hrs</t>
+        </is>
+      </c>
+      <c r="F67" s="16" t="inlineStr">
+        <is>
+          <t>$80</t>
+        </is>
+      </c>
+      <c r="G67" s="14" t="inlineStr">
+        <is>
           <t>1 day</t>
         </is>
       </c>
-      <c r="E67" s="14" t="inlineStr">
-        <is>
-          <t>8 hrs</t>
-        </is>
-      </c>
-      <c r="F67" s="16" t="inlineStr">
-        <is>
-          <t>$160</t>
-        </is>
-      </c>
-      <c r="G67" s="14" t="inlineStr">
-        <is>
-          <t>2 days</t>
-        </is>
-      </c>
       <c r="H67" s="38" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I67" s="34" t="inlineStr"/>
+      <c r="I67" s="33" t="inlineStr">
+        <is>
+          <t>Nginx handles SSL termination</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="B68" s="14" t="inlineStr"/>
       <c r="C68" s="31" t="inlineStr">
         <is>
-          <t>Production environment setup (Docker Compose + Nginx + self-hosted Postgres + Redis on client's server)</t>
+          <t>DB migration strategy (Drizzle migrate on deploy, zero-downtime)</t>
         </is>
       </c>
       <c r="D68" s="14" t="inlineStr">
@@ -3691,148 +3683,76 @@
           <t>1 day</t>
         </is>
       </c>
-      <c r="H68" s="32" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="H68" s="38" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="I68" s="34" t="inlineStr"/>
     </row>
     <row r="69" ht="20" customHeight="1">
-      <c r="B69" s="14" t="inlineStr"/>
-      <c r="C69" s="31" t="inlineStr">
-        <is>
-          <t>Custom domain + SSL (Let's Encrypt via Certbot + Nginx) + env var management</t>
-        </is>
-      </c>
-      <c r="D69" s="14" t="inlineStr">
-        <is>
-          <t>0.5 day</t>
-        </is>
-      </c>
-      <c r="E69" s="14" t="inlineStr">
-        <is>
-          <t>4 hrs</t>
-        </is>
-      </c>
-      <c r="F69" s="16" t="inlineStr">
-        <is>
-          <t>$80</t>
-        </is>
-      </c>
-      <c r="G69" s="14" t="inlineStr">
-        <is>
-          <t>1 day</t>
-        </is>
-      </c>
-      <c r="H69" s="38" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I69" s="33" t="inlineStr">
-        <is>
-          <t>Nginx handles SSL termination</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="20" customHeight="1">
-      <c r="B70" s="14" t="inlineStr"/>
-      <c r="C70" s="31" t="inlineStr">
-        <is>
-          <t>DB migration strategy (Drizzle migrate on deploy, zero-downtime)</t>
-        </is>
-      </c>
-      <c r="D70" s="14" t="inlineStr">
-        <is>
-          <t>0.5 day</t>
-        </is>
-      </c>
-      <c r="E70" s="14" t="inlineStr">
-        <is>
-          <t>4 hrs</t>
-        </is>
-      </c>
-      <c r="F70" s="16" t="inlineStr">
-        <is>
-          <t>$80</t>
-        </is>
-      </c>
-      <c r="G70" s="14" t="inlineStr">
-        <is>
-          <t>1 day</t>
-        </is>
-      </c>
-      <c r="H70" s="38" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I70" s="34" t="inlineStr"/>
-    </row>
-    <row r="71" ht="20" customHeight="1">
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B69" s="8" t="inlineStr">
         <is>
           <t>Phase 7 Total</t>
         </is>
       </c>
-      <c r="C71" s="35" t="inlineStr"/>
-      <c r="D71" s="8" t="inlineStr">
+      <c r="C69" s="35" t="inlineStr"/>
+      <c r="D69" s="8" t="inlineStr">
         <is>
           <t>6.5 days</t>
         </is>
       </c>
-      <c r="E71" s="8" t="inlineStr">
+      <c r="E69" s="8" t="inlineStr">
         <is>
           <t>52 hrs</t>
         </is>
       </c>
-      <c r="F71" s="8" t="inlineStr">
+      <c r="F69" s="8" t="inlineStr">
         <is>
           <t>$1,040</t>
         </is>
       </c>
-      <c r="G71" s="8" t="inlineStr">
+      <c r="G69" s="8" t="inlineStr">
         <is>
           <t>15 days</t>
         </is>
       </c>
-      <c r="H71" s="36" t="inlineStr"/>
-      <c r="I71" s="37" t="inlineStr"/>
-    </row>
-    <row r="72" ht="26" customHeight="1">
-      <c r="B72" s="17" t="inlineStr">
+      <c r="H69" s="36" t="inlineStr"/>
+      <c r="I69" s="37" t="inlineStr"/>
+    </row>
+    <row r="70" ht="26" customHeight="1">
+      <c r="B70" s="17" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C72" s="40" t="inlineStr">
+      <c r="C70" s="40" t="inlineStr">
         <is>
           <t>All Phases (1–7)  ·  556 hrs  ·  $20/hr</t>
         </is>
       </c>
-      <c r="D72" s="17" t="inlineStr">
+      <c r="D70" s="17" t="inlineStr">
         <is>
           <t>69.5 days</t>
         </is>
       </c>
-      <c r="E72" s="17" t="inlineStr">
+      <c r="E70" s="17" t="inlineStr">
         <is>
           <t>556 hrs</t>
         </is>
       </c>
-      <c r="F72" s="17" t="inlineStr">
+      <c r="F70" s="17" t="inlineStr">
         <is>
           <t>$11,120</t>
         </is>
       </c>
-      <c r="G72" s="17" t="inlineStr">
+      <c r="G70" s="17" t="inlineStr">
         <is>
           <t>163 days</t>
         </is>
       </c>
-      <c r="H72" s="36" t="inlineStr"/>
-      <c r="I72" s="33" t="inlineStr">
+      <c r="H70" s="36" t="inlineStr"/>
+      <c r="I70" s="33" t="inlineStr">
         <is>
           <t>Wall-clock: ~3–4 weeks with parallelism</t>
         </is>
@@ -3840,14 +3760,14 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="B56:I56"/>
-    <mergeCell ref="B64:I64"/>
+    <mergeCell ref="B44:I44"/>
+    <mergeCell ref="B62:I62"/>
+    <mergeCell ref="B29:I29"/>
     <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B54:I54"/>
     <mergeCell ref="B22:I22"/>
     <mergeCell ref="B14:I14"/>
     <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B46:I46"/>
     <mergeCell ref="B1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: add server/hardware cost section to estimate Excel
Summary tab now includes three hosting options below the infra table:
- Option A: existing client server ($15–25/mo electricity only)
- Option B: VPS rental — Hetzner CX32 $9/mo (min) / CX42 $19/mo (rec)
- Option C: buy dedicated hardware ($150–900 one-time + electricity)
Recommendation callout highlights Hetzner CX42 if no existing server.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Estimate.xlsx
+++ b/docs/DecisionOS_Estimate.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -99,6 +99,23 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="001B2A4A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="006B7280"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="16"/>
@@ -116,18 +133,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="006B7280"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <color rgb="0092400E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="006B7280"/>
       <sz val="10"/>
     </font>
     <font>
@@ -160,7 +166,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -200,6 +206,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E40AF"/>
       </patternFill>
     </fill>
     <fill>
@@ -259,7 +270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -334,10 +345,38 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -346,13 +385,13 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -361,13 +400,13 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -379,9 +418,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -391,17 +427,17 @@
     <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -409,40 +445,43 @@
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -810,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H38"/>
+  <dimension ref="B1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1571,28 +1610,422 @@
         </is>
       </c>
     </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>SERVER / HARDWARE COST (CLIENT'S HOSTING)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="B42" s="28" t="inlineStr">
+        <is>
+          <t>Minimum specs to run DecisionOS:  4 CPU cores  ·  8 GB RAM (16 GB recommended)  ·  100 GB SSD  ·  100 Mbps upload</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="B43" s="29" t="inlineStr">
+        <is>
+          <t>Option A — Client Already Has a Server  (most likely scenario)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="D44" s="20" t="n"/>
+      <c r="E44" s="20" t="n"/>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>One-Time Cost</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Monthly Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="19" customHeight="1">
+      <c r="B45" s="21" t="inlineStr">
+        <is>
+          <t>Existing server hardware</t>
+        </is>
+      </c>
+      <c r="C45" s="21" t="inlineStr">
+        <is>
+          <t>Already owned by client — no additional purchase needed</t>
+        </is>
+      </c>
+      <c r="D45" s="22" t="n"/>
+      <c r="E45" s="22" t="n"/>
+      <c r="G45" s="23" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="H45" s="16" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="19" customHeight="1">
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>~200 W server running 24/7</t>
+        </is>
+      </c>
+      <c r="D46" s="24" t="n"/>
+      <c r="E46" s="24" t="n"/>
+      <c r="G46" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="16" t="inlineStr">
+        <is>
+          <t>$15–25</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="19" customHeight="1">
+      <c r="B47" s="21" t="inlineStr">
+        <is>
+          <t>Business internet</t>
+        </is>
+      </c>
+      <c r="C47" s="21" t="inlineStr">
+        <is>
+          <t>For API access + CI/CD deploys (if not already in place)</t>
+        </is>
+      </c>
+      <c r="D47" s="22" t="n"/>
+      <c r="E47" s="22" t="n"/>
+      <c r="G47" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" s="16" t="inlineStr">
+        <is>
+          <t>$50–100</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="19" customHeight="1">
+      <c r="B48" s="18" t="inlineStr">
+        <is>
+          <t>TOTAL (Option A)</t>
+        </is>
+      </c>
+      <c r="C48" s="25" t="inlineStr"/>
+      <c r="D48" s="26" t="n"/>
+      <c r="E48" s="26" t="n"/>
+      <c r="G48" s="17" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="H48" s="17" t="inlineStr">
+        <is>
+          <t>$15–25/month</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="B50" s="29" t="inlineStr">
+        <is>
+          <t>Option B — Rent a VPS  (if no existing server)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Provider / Plan</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Spec</t>
+        </is>
+      </c>
+      <c r="D51" s="20" t="n"/>
+      <c r="E51" s="20" t="n"/>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Monthly Cost</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="19" customHeight="1">
+      <c r="B52" s="21" t="inlineStr">
+        <is>
+          <t>Hetzner Cloud CX32  ⭐ Min</t>
+        </is>
+      </c>
+      <c r="C52" s="21" t="inlineStr">
+        <is>
+          <t>4 vCPU · 8 GB RAM · 80 GB SSD</t>
+        </is>
+      </c>
+      <c r="D52" s="22" t="n"/>
+      <c r="E52" s="22" t="n"/>
+      <c r="G52" s="23" t="inlineStr">
+        <is>
+          <t>~$9/mo</t>
+        </is>
+      </c>
+      <c r="H52" s="30" t="inlineStr">
+        <is>
+          <t>Best value for minimum viable</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="19" customHeight="1">
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Hetzner Cloud CX42  ⭐ Rec</t>
+        </is>
+      </c>
+      <c r="C53" s="31" t="inlineStr">
+        <is>
+          <t>8 vCPU · 16 GB RAM · 160 GB SSD</t>
+        </is>
+      </c>
+      <c r="D53" s="32" t="n"/>
+      <c r="E53" s="32" t="n"/>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>~$19/mo</t>
+        </is>
+      </c>
+      <c r="H53" s="33" t="inlineStr">
+        <is>
+          <t>Recommended — pgvector headroom</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="19" customHeight="1">
+      <c r="B54" s="21" t="inlineStr">
+        <is>
+          <t>OVH VPS Value</t>
+        </is>
+      </c>
+      <c r="C54" s="21" t="inlineStr">
+        <is>
+          <t>4 vCPU · 8 GB RAM · 80 GB SSD</t>
+        </is>
+      </c>
+      <c r="D54" s="22" t="n"/>
+      <c r="E54" s="22" t="n"/>
+      <c r="G54" s="23" t="inlineStr">
+        <is>
+          <t>~$12/mo</t>
+        </is>
+      </c>
+      <c r="H54" s="30" t="inlineStr">
+        <is>
+          <t>EU-based alternative</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="19" customHeight="1">
+      <c r="B55" s="15" t="inlineStr">
+        <is>
+          <t>DigitalOcean Droplet</t>
+        </is>
+      </c>
+      <c r="C55" s="15" t="inlineStr">
+        <is>
+          <t>4 vCPU · 8 GB RAM · 160 GB SSD</t>
+        </is>
+      </c>
+      <c r="D55" s="24" t="n"/>
+      <c r="E55" s="24" t="n"/>
+      <c r="G55" s="14" t="inlineStr">
+        <is>
+          <t>$48/mo</t>
+        </is>
+      </c>
+      <c r="H55" s="34" t="inlineStr">
+        <is>
+          <t>Reliable but 5× more than Hetzner</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="B57" s="29" t="inlineStr">
+        <is>
+          <t>Option C — Buy Dedicated Hardware  (one-time purchase)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Spec</t>
+        </is>
+      </c>
+      <c r="D58" s="20" t="n"/>
+      <c r="E58" s="20" t="n"/>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>One-Time Cost</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Monthly (electricity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="19" customHeight="1">
+      <c r="B59" s="21" t="inlineStr">
+        <is>
+          <t>Refurbished Dell PowerEdge R220</t>
+        </is>
+      </c>
+      <c r="C59" s="21" t="inlineStr">
+        <is>
+          <t>4 core · 16 GB RAM · 1 TB HDD</t>
+        </is>
+      </c>
+      <c r="D59" s="22" t="n"/>
+      <c r="E59" s="22" t="n"/>
+      <c r="G59" s="23" t="inlineStr">
+        <is>
+          <t>$150–250</t>
+        </is>
+      </c>
+      <c r="H59" s="35" t="inlineStr">
+        <is>
+          <t>$15–25</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="19" customHeight="1">
+      <c r="B60" s="15" t="inlineStr">
+        <is>
+          <t>Mini PC (Beelink / Intel NUC)</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>4 core · 16 GB RAM · 512 GB SSD</t>
+        </is>
+      </c>
+      <c r="D60" s="24" t="n"/>
+      <c r="E60" s="24" t="n"/>
+      <c r="G60" s="14" t="inlineStr">
+        <is>
+          <t>$200–350</t>
+        </is>
+      </c>
+      <c r="H60" s="36" t="inlineStr">
+        <is>
+          <t>$10–15</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="19" customHeight="1">
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>New small-form server  ⭐ Rec</t>
+        </is>
+      </c>
+      <c r="C61" s="31" t="inlineStr">
+        <is>
+          <t>8 core · 32 GB RAM · 1 TB SSD</t>
+        </is>
+      </c>
+      <c r="D61" s="32" t="n"/>
+      <c r="E61" s="32" t="n"/>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>$600–900</t>
+        </is>
+      </c>
+      <c r="H61" s="37" t="inlineStr">
+        <is>
+          <t>$20–30</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="B63" s="19" t="inlineStr">
+        <is>
+          <t>Recommendation: If client has an existing server → use it ($0 extra). If not → Hetzner CX42 (~$19/mo) gives 16 GB RAM headroom for pgvector at minimal cost.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="40">
+    <mergeCell ref="C54:E54"/>
     <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C44:E44"/>
+    <mergeCell ref="C55:E55"/>
     <mergeCell ref="C9:H9"/>
     <mergeCell ref="C38:F38"/>
     <mergeCell ref="B30:H30"/>
     <mergeCell ref="C32:F32"/>
     <mergeCell ref="C12:H12"/>
+    <mergeCell ref="C59:E59"/>
     <mergeCell ref="C37:F37"/>
     <mergeCell ref="B5:H5"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="C46:E46"/>
+    <mergeCell ref="B63:H63"/>
     <mergeCell ref="C11:H11"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="B50:H50"/>
+    <mergeCell ref="B41:H41"/>
+    <mergeCell ref="C52:E52"/>
     <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="C48:E48"/>
     <mergeCell ref="C8:H8"/>
     <mergeCell ref="B16:H16"/>
     <mergeCell ref="C33:F33"/>
     <mergeCell ref="C7:H7"/>
     <mergeCell ref="C35:F35"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="B43:H43"/>
+    <mergeCell ref="B42:H42"/>
+    <mergeCell ref="C58:E58"/>
     <mergeCell ref="C6:H6"/>
     <mergeCell ref="C31:F31"/>
     <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B57:H57"/>
+    <mergeCell ref="C45:E45"/>
     <mergeCell ref="C36:F36"/>
     <mergeCell ref="B28:H28"/>
+    <mergeCell ref="C47:E47"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1620,14 +2053,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="50" customHeight="1">
-      <c r="B1" s="28" t="inlineStr">
+      <c r="B1" s="38" t="inlineStr">
         <is>
           <t>DecisionOS — Detailed Phase Estimate</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="B2" s="29" t="inlineStr">
+      <c r="B2" s="39" t="inlineStr">
         <is>
           <t>Rate: $20/hr × 8 hrs/day = $160/day. AI-assisted (Claude Code SDD). Traditional equivalent shown for comparison.</t>
         </is>
@@ -1676,7 +2109,7 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="30" t="inlineStr">
+      <c r="B5" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Phase 1  —  Backend Foundation</t>
         </is>
@@ -1684,7 +2117,7 @@
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="B6" s="14" t="inlineStr"/>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="C6" s="41" t="inlineStr">
         <is>
           <t>PostgreSQL schema (all 7 table groups: identity, data, BI, AI/chat, decisions, workflow, governance)</t>
         </is>
@@ -1709,12 +2142,12 @@
           <t>4 days</t>
         </is>
       </c>
-      <c r="H6" s="32" t="inlineStr">
+      <c r="H6" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I6" s="33" t="inlineStr">
+      <c r="I6" s="43" t="inlineStr">
         <is>
           <t>Drizzle ORM + self-hosted Postgres</t>
         </is>
@@ -1722,7 +2155,7 @@
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="B7" s="14" t="inlineStr"/>
-      <c r="C7" s="31" t="inlineStr">
+      <c r="C7" s="41" t="inlineStr">
         <is>
           <t>Self-hosted Postgres setup + pgvector extension + Drizzle migrations</t>
         </is>
@@ -1747,12 +2180,12 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H7" s="32" t="inlineStr">
+      <c r="H7" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I7" s="33" t="inlineStr">
+      <c r="I7" s="43" t="inlineStr">
         <is>
           <t>Runs on client's server</t>
         </is>
@@ -1760,7 +2193,7 @@
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="B8" s="14" t="inlineStr"/>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="C8" s="41" t="inlineStr">
         <is>
           <t>Auth.js v5 — Credentials + bcrypt + JWT (httpOnly cookie, 7-day)</t>
         </is>
@@ -1785,16 +2218,16 @@
           <t>4 days</t>
         </is>
       </c>
-      <c r="H8" s="32" t="inlineStr">
+      <c r="H8" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I8" s="34" t="inlineStr"/>
+      <c r="I8" s="44" t="inlineStr"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="B9" s="14" t="inlineStr"/>
-      <c r="C9" s="31" t="inlineStr">
+      <c r="C9" s="41" t="inlineStr">
         <is>
           <t>Session middleware (JWT validation on every API route)</t>
         </is>
@@ -1819,16 +2252,16 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H9" s="32" t="inlineStr">
+      <c r="H9" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I9" s="34" t="inlineStr"/>
+      <c r="I9" s="44" t="inlineStr"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="B10" s="14" t="inlineStr"/>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="C10" s="41" t="inlineStr">
         <is>
           <t>Schema-per-tenant middleware (search_path per connection)</t>
         </is>
@@ -1853,12 +2286,12 @@
           <t>4 days</t>
         </is>
       </c>
-      <c r="H10" s="32" t="inlineStr">
+      <c r="H10" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I10" s="33" t="inlineStr">
+      <c r="I10" s="43" t="inlineStr">
         <is>
           <t>Complete tenant isolation at DB level</t>
         </is>
@@ -1866,7 +2299,7 @@
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="B11" s="14" t="inlineStr"/>
-      <c r="C11" s="31" t="inlineStr">
+      <c r="C11" s="41" t="inlineStr">
         <is>
           <t>Next.js API Routes scaffold (versioned, Zod-typed)</t>
         </is>
@@ -1891,16 +2324,16 @@
           <t>3 days</t>
         </is>
       </c>
-      <c r="H11" s="32" t="inlineStr">
+      <c r="H11" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I11" s="34" t="inlineStr"/>
+      <c r="I11" s="44" t="inlineStr"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="B12" s="14" t="inlineStr"/>
-      <c r="C12" s="31" t="inlineStr">
+      <c r="C12" s="41" t="inlineStr">
         <is>
           <t>Zustand auth store → real JWT session (replace mock cookie)</t>
         </is>
@@ -1925,12 +2358,12 @@
           <t>1 day</t>
         </is>
       </c>
-      <c r="H12" s="32" t="inlineStr">
+      <c r="H12" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I12" s="34" t="inlineStr"/>
+      <c r="I12" s="44" t="inlineStr"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="B13" s="8" t="inlineStr">
@@ -1938,7 +2371,7 @@
           <t>Phase 1 Total</t>
         </is>
       </c>
-      <c r="C13" s="35" t="inlineStr"/>
+      <c r="C13" s="45" t="inlineStr"/>
       <c r="D13" s="8" t="inlineStr">
         <is>
           <t>7.5 days</t>
@@ -1959,11 +2392,11 @@
           <t>20 days</t>
         </is>
       </c>
-      <c r="H13" s="36" t="inlineStr"/>
-      <c r="I13" s="37" t="inlineStr"/>
+      <c r="H13" s="46" t="inlineStr"/>
+      <c r="I13" s="47" t="inlineStr"/>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B14" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Phase 2  —  File Ingestion Pipeline</t>
         </is>
@@ -1971,7 +2404,7 @@
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="B15" s="14" t="inlineStr"/>
-      <c r="C15" s="31" t="inlineStr">
+      <c r="C15" s="41" t="inlineStr">
         <is>
           <t>File upload endpoint (multipart → local disk, served via Nginx static path)</t>
         </is>
@@ -1996,16 +2429,16 @@
           <t>3 days</t>
         </is>
       </c>
-      <c r="H15" s="38" t="inlineStr">
+      <c r="H15" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I15" s="34" t="inlineStr"/>
+      <c r="I15" s="44" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="14" t="inlineStr"/>
-      <c r="C16" s="31" t="inlineStr">
+      <c r="C16" s="41" t="inlineStr">
         <is>
           <t>CSV parser (Papa Parse) + Excel parser (xlsx library)</t>
         </is>
@@ -2030,16 +2463,16 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H16" s="38" t="inlineStr">
+      <c r="H16" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I16" s="34" t="inlineStr"/>
+      <c r="I16" s="44" t="inlineStr"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="14" t="inlineStr"/>
-      <c r="C17" s="31" t="inlineStr">
+      <c r="C17" s="41" t="inlineStr">
         <is>
           <t>Schema inference (auto-detect column names + data types)</t>
         </is>
@@ -2064,16 +2497,16 @@
           <t>4 days</t>
         </is>
       </c>
-      <c r="H17" s="38" t="inlineStr">
+      <c r="H17" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I17" s="34" t="inlineStr"/>
+      <c r="I17" s="44" t="inlineStr"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="B18" s="14" t="inlineStr"/>
-      <c r="C18" s="31" t="inlineStr">
+      <c r="C18" s="41" t="inlineStr">
         <is>
           <t>Data normalisation → typed Postgres tables per source (dynamic DDL)</t>
         </is>
@@ -2098,16 +2531,16 @@
           <t>3 days</t>
         </is>
       </c>
-      <c r="H18" s="38" t="inlineStr">
+      <c r="H18" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I18" s="34" t="inlineStr"/>
+      <c r="I18" s="44" t="inlineStr"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="B19" s="14" t="inlineStr"/>
-      <c r="C19" s="31" t="inlineStr">
+      <c r="C19" s="41" t="inlineStr">
         <is>
           <t>Upload wizard → real API integration (existing frontend)</t>
         </is>
@@ -2132,16 +2565,16 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H19" s="38" t="inlineStr">
+      <c r="H19" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I19" s="34" t="inlineStr"/>
+      <c r="I19" s="44" t="inlineStr"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="B20" s="14" t="inlineStr"/>
-      <c r="C20" s="31" t="inlineStr">
+      <c r="C20" s="41" t="inlineStr">
         <is>
           <t>Ingestion history logging</t>
         </is>
@@ -2166,12 +2599,12 @@
           <t>1 day</t>
         </is>
       </c>
-      <c r="H20" s="39" t="inlineStr">
+      <c r="H20" s="49" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I20" s="34" t="inlineStr"/>
+      <c r="I20" s="44" t="inlineStr"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="B21" s="8" t="inlineStr">
@@ -2179,7 +2612,7 @@
           <t>Phase 2 Total</t>
         </is>
       </c>
-      <c r="C21" s="35" t="inlineStr"/>
+      <c r="C21" s="45" t="inlineStr"/>
       <c r="D21" s="8" t="inlineStr">
         <is>
           <t>6.5 days</t>
@@ -2200,11 +2633,11 @@
           <t>15 days</t>
         </is>
       </c>
-      <c r="H21" s="36" t="inlineStr"/>
-      <c r="I21" s="37" t="inlineStr"/>
+      <c r="H21" s="46" t="inlineStr"/>
+      <c r="I21" s="47" t="inlineStr"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="30" t="inlineStr">
+      <c r="B22" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Phase 3  —  Data Connectors</t>
         </is>
@@ -2212,7 +2645,7 @@
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="B23" s="14" t="inlineStr"/>
-      <c r="C23" s="31" t="inlineStr">
+      <c r="C23" s="41" t="inlineStr">
         <is>
           <t>Zoho CRM — OAuth 2.0, REST API v7, Contacts/Deals/Accounts sync, delta sync via Modified_Time</t>
         </is>
@@ -2242,7 +2675,7 @@
           <t>Launch</t>
         </is>
       </c>
-      <c r="I23" s="33" t="inlineStr">
+      <c r="I23" s="43" t="inlineStr">
         <is>
           <t>Client to register Zoho Server App</t>
         </is>
@@ -2250,7 +2683,7 @@
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="B24" s="14" t="inlineStr"/>
-      <c r="C24" s="31" t="inlineStr">
+      <c r="C24" s="41" t="inlineStr">
         <is>
           <t>Custom ERP — Generic REST adapter, configurable auth, field mapping UI, webhook receiver</t>
         </is>
@@ -2280,7 +2713,7 @@
           <t>Launch</t>
         </is>
       </c>
-      <c r="I24" s="33" t="inlineStr">
+      <c r="I24" s="43" t="inlineStr">
         <is>
           <t>Client to share API docs</t>
         </is>
@@ -2288,7 +2721,7 @@
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="B25" s="14" t="inlineStr"/>
-      <c r="C25" s="31" t="inlineStr">
+      <c r="C25" s="41" t="inlineStr">
         <is>
           <t>PostgreSQL direct — connection config, table browser, scheduled SELECT pull</t>
         </is>
@@ -2318,11 +2751,11 @@
           <t>Launch</t>
         </is>
       </c>
-      <c r="I25" s="34" t="inlineStr"/>
+      <c r="I25" s="44" t="inlineStr"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="B26" s="14" t="inlineStr"/>
-      <c r="C26" s="31" t="inlineStr">
+      <c r="C26" s="41" t="inlineStr">
         <is>
           <t>Sync scheduler — pg-boss job queue, cron per source, retry + exponential backoff</t>
         </is>
@@ -2352,11 +2785,11 @@
           <t>Launch</t>
         </is>
       </c>
-      <c r="I26" s="34" t="inlineStr"/>
+      <c r="I26" s="44" t="inlineStr"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="B27" s="14" t="inlineStr"/>
-      <c r="C27" s="31" t="inlineStr">
+      <c r="C27" s="41" t="inlineStr">
         <is>
           <t>Connector UI wiring — OAuth redirect → callback → encrypted credential storage (AES-256-GCM)</t>
         </is>
@@ -2386,7 +2819,7 @@
           <t>Launch</t>
         </is>
       </c>
-      <c r="I27" s="34" t="inlineStr"/>
+      <c r="I27" s="44" t="inlineStr"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="B28" s="8" t="inlineStr">
@@ -2394,7 +2827,7 @@
           <t>Phase 3 Total</t>
         </is>
       </c>
-      <c r="C28" s="35" t="inlineStr"/>
+      <c r="C28" s="45" t="inlineStr"/>
       <c r="D28" s="8" t="inlineStr">
         <is>
           <t>13 days</t>
@@ -2415,11 +2848,11 @@
           <t>28 days</t>
         </is>
       </c>
-      <c r="H28" s="36" t="inlineStr"/>
-      <c r="I28" s="37" t="inlineStr"/>
+      <c r="H28" s="46" t="inlineStr"/>
+      <c r="I28" s="47" t="inlineStr"/>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="B29" s="30" t="inlineStr">
+      <c r="B29" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Phase 4  —  AI / LLM Engine</t>
         </is>
@@ -2427,7 +2860,7 @@
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="B30" s="14" t="inlineStr"/>
-      <c r="C30" s="31" t="inlineStr">
+      <c r="C30" s="41" t="inlineStr">
         <is>
           <t>pgvector extension + embedding schema</t>
         </is>
@@ -2452,16 +2885,16 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H30" s="32" t="inlineStr">
+      <c r="H30" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I30" s="34" t="inlineStr"/>
+      <c r="I30" s="44" t="inlineStr"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="B31" s="14" t="inlineStr"/>
-      <c r="C31" s="31" t="inlineStr">
+      <c r="C31" s="41" t="inlineStr">
         <is>
           <t>Embedding pipeline — chunk rows → embed via provider → store vectors</t>
         </is>
@@ -2486,16 +2919,16 @@
           <t>5 days</t>
         </is>
       </c>
-      <c r="H31" s="32" t="inlineStr">
+      <c r="H31" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I31" s="34" t="inlineStr"/>
+      <c r="I31" s="44" t="inlineStr"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="B32" s="14" t="inlineStr"/>
-      <c r="C32" s="31" t="inlineStr">
+      <c r="C32" s="41" t="inlineStr">
         <is>
           <t>RAG retrieval — query → embed → cosine similarity → context assembly</t>
         </is>
@@ -2520,16 +2953,16 @@
           <t>6 days</t>
         </is>
       </c>
-      <c r="H32" s="32" t="inlineStr">
+      <c r="H32" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I32" s="34" t="inlineStr"/>
+      <c r="I32" s="44" t="inlineStr"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="B33" s="14" t="inlineStr"/>
-      <c r="C33" s="31" t="inlineStr">
+      <c r="C33" s="41" t="inlineStr">
         <is>
           <t>SQL generation — LLM → SQL → AST safety check (SELECT-only) → execute → citations</t>
         </is>
@@ -2554,12 +2987,12 @@
           <t>5 days</t>
         </is>
       </c>
-      <c r="H33" s="32" t="inlineStr">
+      <c r="H33" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I33" s="33" t="inlineStr">
+      <c r="I33" s="43" t="inlineStr">
         <is>
           <t>node-sql-parser prevents writes</t>
         </is>
@@ -2567,7 +3000,7 @@
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="B34" s="14" t="inlineStr"/>
-      <c r="C34" s="31" t="inlineStr">
+      <c r="C34" s="41" t="inlineStr">
         <is>
           <t>Multi-provider LLM router — routes to tenant's configured provider</t>
         </is>
@@ -2592,16 +3025,16 @@
           <t>4 days</t>
         </is>
       </c>
-      <c r="H34" s="32" t="inlineStr">
+      <c r="H34" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I34" s="34" t="inlineStr"/>
+      <c r="I34" s="44" t="inlineStr"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="B35" s="14" t="inlineStr"/>
-      <c r="C35" s="31" t="inlineStr">
+      <c r="C35" s="41" t="inlineStr">
         <is>
           <t>LLM provider integrations: Anthropic Claude, OpenAI GPT-4o, Google Gemini</t>
         </is>
@@ -2626,12 +3059,12 @@
           <t>5 days</t>
         </is>
       </c>
-      <c r="H35" s="32" t="inlineStr">
+      <c r="H35" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I35" s="33" t="inlineStr">
+      <c r="I35" s="43" t="inlineStr">
         <is>
           <t>Tenant supplies own API keys</t>
         </is>
@@ -2639,7 +3072,7 @@
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="B36" s="14" t="inlineStr"/>
-      <c r="C36" s="31" t="inlineStr">
+      <c r="C36" s="41" t="inlineStr">
         <is>
           <t>LLM Connect wizard — provider selector → paste API key → test connection → save default</t>
         </is>
@@ -2664,12 +3097,12 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H36" s="38" t="inlineStr">
+      <c r="H36" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I36" s="33" t="inlineStr">
+      <c r="I36" s="43" t="inlineStr">
         <is>
           <t>Simple wizard-style UX</t>
         </is>
@@ -2677,7 +3110,7 @@
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="B37" s="14" t="inlineStr"/>
-      <c r="C37" s="31" t="inlineStr">
+      <c r="C37" s="41" t="inlineStr">
         <is>
           <t>LLM usage logging — llm_usage_logs table (tokens, cost_estimate, provider, user)</t>
         </is>
@@ -2702,12 +3135,12 @@
           <t>1 day</t>
         </is>
       </c>
-      <c r="H37" s="38" t="inlineStr">
+      <c r="H37" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I37" s="33" t="inlineStr">
+      <c r="I37" s="43" t="inlineStr">
         <is>
           <t>Foundation for usage dashboard</t>
         </is>
@@ -2715,7 +3148,7 @@
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="B38" s="14" t="inlineStr"/>
-      <c r="C38" s="31" t="inlineStr">
+      <c r="C38" s="41" t="inlineStr">
         <is>
           <t>7-agent orchestration — Intent → Governance (PII masking) → Data Analyst → BI → Insight → Recommendation → Workflow</t>
         </is>
@@ -2740,12 +3173,12 @@
           <t>9 days</t>
         </is>
       </c>
-      <c r="H38" s="32" t="inlineStr">
+      <c r="H38" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I38" s="33" t="inlineStr">
+      <c r="I38" s="43" t="inlineStr">
         <is>
           <t>Strong model for analyst/insight/rec; fast for others</t>
         </is>
@@ -2753,7 +3186,7 @@
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="B39" s="14" t="inlineStr"/>
-      <c r="C39" s="31" t="inlineStr">
+      <c r="C39" s="41" t="inlineStr">
         <is>
           <t>Chat session persistence — chat_sessions + chat_messages CRUD API, session list, pagination</t>
         </is>
@@ -2778,12 +3211,12 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H39" s="32" t="inlineStr">
+      <c r="H39" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I39" s="33" t="inlineStr">
+      <c r="I39" s="43" t="inlineStr">
         <is>
           <t>Feeds session sidebar</t>
         </is>
@@ -2791,7 +3224,7 @@
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="B40" s="14" t="inlineStr"/>
-      <c r="C40" s="31" t="inlineStr">
+      <c r="C40" s="41" t="inlineStr">
         <is>
           <t>SSE streaming — AI response streams token-by-token to chat UI</t>
         </is>
@@ -2816,16 +3249,16 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H40" s="32" t="inlineStr">
+      <c r="H40" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I40" s="34" t="inlineStr"/>
+      <c r="I40" s="44" t="inlineStr"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="B41" s="14" t="inlineStr"/>
-      <c r="C41" s="31" t="inlineStr">
+      <c r="C41" s="41" t="inlineStr">
         <is>
           <t>AI Executive Summary generator — nightly cron per tenant</t>
         </is>
@@ -2850,16 +3283,16 @@
           <t>3 days</t>
         </is>
       </c>
-      <c r="H41" s="39" t="inlineStr">
+      <c r="H41" s="49" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I41" s="34" t="inlineStr"/>
+      <c r="I41" s="44" t="inlineStr"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="14" t="inlineStr"/>
-      <c r="C42" s="31" t="inlineStr">
+      <c r="C42" s="41" t="inlineStr">
         <is>
           <t>Insight + Recommendation auto-generation (LLM + threshold rule engine, 4h cron)</t>
         </is>
@@ -2884,12 +3317,12 @@
           <t>5 days</t>
         </is>
       </c>
-      <c r="H42" s="38" t="inlineStr">
+      <c r="H42" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I42" s="34" t="inlineStr"/>
+      <c r="I42" s="44" t="inlineStr"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="B43" s="8" t="inlineStr">
@@ -2897,7 +3330,7 @@
           <t>Phase 4 Total</t>
         </is>
       </c>
-      <c r="C43" s="35" t="inlineStr"/>
+      <c r="C43" s="45" t="inlineStr"/>
       <c r="D43" s="8" t="inlineStr">
         <is>
           <t>21 days</t>
@@ -2918,11 +3351,11 @@
           <t>51 days</t>
         </is>
       </c>
-      <c r="H43" s="36" t="inlineStr"/>
-      <c r="I43" s="37" t="inlineStr"/>
+      <c r="H43" s="46" t="inlineStr"/>
+      <c r="I43" s="47" t="inlineStr"/>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="B44" s="30" t="inlineStr">
+      <c r="B44" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Phase 5  —  Frontend Integration + Subscription Enforcement</t>
         </is>
@@ -2930,7 +3363,7 @@
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="B45" s="14" t="inlineStr"/>
-      <c r="C45" s="31" t="inlineStr">
+      <c r="C45" s="41" t="inlineStr">
         <is>
           <t>TanStack Query hooks for all endpoints (users, KPIs, insights, recommendations, tasks)</t>
         </is>
@@ -2955,16 +3388,16 @@
           <t>4 days</t>
         </is>
       </c>
-      <c r="H45" s="32" t="inlineStr">
+      <c r="H45" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I45" s="34" t="inlineStr"/>
+      <c r="I45" s="44" t="inlineStr"/>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="B46" s="14" t="inlineStr"/>
-      <c r="C46" s="31" t="inlineStr">
+      <c r="C46" s="41" t="inlineStr">
         <is>
           <t>Real KPI computation (SQL aggregates per tenant, configurable formulas)</t>
         </is>
@@ -2989,16 +3422,16 @@
           <t>4 days</t>
         </is>
       </c>
-      <c r="H46" s="38" t="inlineStr">
+      <c r="H46" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I46" s="34" t="inlineStr"/>
+      <c r="I46" s="44" t="inlineStr"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="B47" s="14" t="inlineStr"/>
-      <c r="C47" s="31" t="inlineStr">
+      <c r="C47" s="41" t="inlineStr">
         <is>
           <t>Real dashboard charts (live data → Recharts via API)</t>
         </is>
@@ -3023,16 +3456,16 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H47" s="38" t="inlineStr">
+      <c r="H47" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I47" s="34" t="inlineStr"/>
+      <c r="I47" s="44" t="inlineStr"/>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="B48" s="14" t="inlineStr"/>
-      <c r="C48" s="31" t="inlineStr">
+      <c r="C48" s="41" t="inlineStr">
         <is>
           <t>Notification system (SSE endpoint → existing notification bell)</t>
         </is>
@@ -3057,16 +3490,16 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H48" s="39" t="inlineStr">
+      <c r="H48" s="49" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I48" s="34" t="inlineStr"/>
+      <c r="I48" s="44" t="inlineStr"/>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="B49" s="14" t="inlineStr"/>
-      <c r="C49" s="31" t="inlineStr">
+      <c r="C49" s="41" t="inlineStr">
         <is>
           <t>Workflow / task CRUD persistence</t>
         </is>
@@ -3091,16 +3524,16 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H49" s="39" t="inlineStr">
+      <c r="H49" s="49" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I49" s="34" t="inlineStr"/>
+      <c r="I49" s="44" t="inlineStr"/>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="B50" s="14" t="inlineStr"/>
-      <c r="C50" s="31" t="inlineStr">
+      <c r="C50" s="41" t="inlineStr">
         <is>
           <t>Subscription enforcement middleware — user + data source limits → 402 on breach</t>
         </is>
@@ -3125,12 +3558,12 @@
           <t>3 days</t>
         </is>
       </c>
-      <c r="H50" s="38" t="inlineStr">
+      <c r="H50" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I50" s="33" t="inlineStr">
+      <c r="I50" s="43" t="inlineStr">
         <is>
           <t>No query cap — tenant pays own LLM</t>
         </is>
@@ -3138,7 +3571,7 @@
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="B51" s="14" t="inlineStr"/>
-      <c r="C51" s="31" t="inlineStr">
+      <c r="C51" s="41" t="inlineStr">
         <is>
           <t>Tenant Admin Console — LLM wizard + usage dashboard (tokens, cost estimate, per-user)</t>
         </is>
@@ -3163,16 +3596,16 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H51" s="38" t="inlineStr">
+      <c r="H51" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I51" s="34" t="inlineStr"/>
+      <c r="I51" s="44" t="inlineStr"/>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="B52" s="14" t="inlineStr"/>
-      <c r="C52" s="31" t="inlineStr">
+      <c r="C52" s="41" t="inlineStr">
         <is>
           <t>Platform Admin panel — plan CRUD, per-tenant plan assignment</t>
         </is>
@@ -3197,12 +3630,12 @@
           <t>1 day</t>
         </is>
       </c>
-      <c r="H52" s="38" t="inlineStr">
+      <c r="H52" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I52" s="34" t="inlineStr"/>
+      <c r="I52" s="44" t="inlineStr"/>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="B53" s="8" t="inlineStr">
@@ -3210,7 +3643,7 @@
           <t>Phase 5 Total</t>
         </is>
       </c>
-      <c r="C53" s="35" t="inlineStr"/>
+      <c r="C53" s="45" t="inlineStr"/>
       <c r="D53" s="8" t="inlineStr">
         <is>
           <t>9.5 days</t>
@@ -3231,11 +3664,11 @@
           <t>20 days</t>
         </is>
       </c>
-      <c r="H53" s="36" t="inlineStr"/>
-      <c r="I53" s="37" t="inlineStr"/>
+      <c r="H53" s="46" t="inlineStr"/>
+      <c r="I53" s="47" t="inlineStr"/>
     </row>
     <row r="54" ht="20" customHeight="1">
-      <c r="B54" s="30" t="inlineStr">
+      <c r="B54" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Phase 6  —  Production Hardening</t>
         </is>
@@ -3243,7 +3676,7 @@
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="B55" s="14" t="inlineStr"/>
-      <c r="C55" s="31" t="inlineStr">
+      <c r="C55" s="41" t="inlineStr">
         <is>
           <t>API rate limiting (self-hosted Redis sliding window, per user + per tenant)</t>
         </is>
@@ -3268,16 +3701,16 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H55" s="38" t="inlineStr">
+      <c r="H55" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I55" s="34" t="inlineStr"/>
+      <c r="I55" s="44" t="inlineStr"/>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="B56" s="14" t="inlineStr"/>
-      <c r="C56" s="31" t="inlineStr">
+      <c r="C56" s="41" t="inlineStr">
         <is>
           <t>Error boundaries + structured logging (Sentry + Pino)</t>
         </is>
@@ -3302,16 +3735,16 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H56" s="38" t="inlineStr">
+      <c r="H56" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I56" s="34" t="inlineStr"/>
+      <c r="I56" s="44" t="inlineStr"/>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="B57" s="14" t="inlineStr"/>
-      <c r="C57" s="31" t="inlineStr">
+      <c r="C57" s="41" t="inlineStr">
         <is>
           <t>Query result caching (self-hosted Redis, 5-min TTL for repeated AI queries)</t>
         </is>
@@ -3336,16 +3769,16 @@
           <t>3 days</t>
         </is>
       </c>
-      <c r="H57" s="39" t="inlineStr">
+      <c r="H57" s="49" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I57" s="34" t="inlineStr"/>
+      <c r="I57" s="44" t="inlineStr"/>
     </row>
     <row r="58" ht="20" customHeight="1">
       <c r="B58" s="14" t="inlineStr"/>
-      <c r="C58" s="31" t="inlineStr">
+      <c r="C58" s="41" t="inlineStr">
         <is>
           <t>Security audit — SQL injection, XSS, OWASP headers, CSRF</t>
         </is>
@@ -3370,16 +3803,16 @@
           <t>3 days</t>
         </is>
       </c>
-      <c r="H58" s="38" t="inlineStr">
+      <c r="H58" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I58" s="34" t="inlineStr"/>
+      <c r="I58" s="44" t="inlineStr"/>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="B59" s="14" t="inlineStr"/>
-      <c r="C59" s="31" t="inlineStr">
+      <c r="C59" s="41" t="inlineStr">
         <is>
           <t>Multi-tenant data isolation audit — cross-tenant pen-test</t>
         </is>
@@ -3404,16 +3837,16 @@
           <t>3 days</t>
         </is>
       </c>
-      <c r="H59" s="32" t="inlineStr">
+      <c r="H59" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I59" s="34" t="inlineStr"/>
+      <c r="I59" s="44" t="inlineStr"/>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="B60" s="14" t="inlineStr"/>
-      <c r="C60" s="31" t="inlineStr">
+      <c r="C60" s="41" t="inlineStr">
         <is>
           <t>Password policy + account lockout</t>
         </is>
@@ -3438,12 +3871,12 @@
           <t>1 day</t>
         </is>
       </c>
-      <c r="H60" s="38" t="inlineStr">
+      <c r="H60" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I60" s="34" t="inlineStr"/>
+      <c r="I60" s="44" t="inlineStr"/>
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="B61" s="8" t="inlineStr">
@@ -3451,7 +3884,7 @@
           <t>Phase 6 Total</t>
         </is>
       </c>
-      <c r="C61" s="35" t="inlineStr"/>
+      <c r="C61" s="45" t="inlineStr"/>
       <c r="D61" s="8" t="inlineStr">
         <is>
           <t>5 days</t>
@@ -3472,11 +3905,11 @@
           <t>14 days</t>
         </is>
       </c>
-      <c r="H61" s="36" t="inlineStr"/>
-      <c r="I61" s="37" t="inlineStr"/>
+      <c r="H61" s="46" t="inlineStr"/>
+      <c r="I61" s="47" t="inlineStr"/>
     </row>
     <row r="62" ht="20" customHeight="1">
-      <c r="B62" s="30" t="inlineStr">
+      <c r="B62" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  Phase 7  —  QA, CI/CD &amp; Deployment</t>
         </is>
@@ -3484,7 +3917,7 @@
     </row>
     <row r="63" ht="20" customHeight="1">
       <c r="B63" s="14" t="inlineStr"/>
-      <c r="C63" s="31" t="inlineStr">
+      <c r="C63" s="41" t="inlineStr">
         <is>
           <t>Unit + integration tests (Vitest — API routes, auth, data ingestion, LLM router)</t>
         </is>
@@ -3509,16 +3942,16 @@
           <t>5 days</t>
         </is>
       </c>
-      <c r="H63" s="38" t="inlineStr">
+      <c r="H63" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I63" s="34" t="inlineStr"/>
+      <c r="I63" s="44" t="inlineStr"/>
     </row>
     <row r="64" ht="20" customHeight="1">
       <c r="B64" s="14" t="inlineStr"/>
-      <c r="C64" s="31" t="inlineStr">
+      <c r="C64" s="41" t="inlineStr">
         <is>
           <t>E2E tests (Playwright — login, upload CSV, Zoho connect, ask AI, workflow create)</t>
         </is>
@@ -3543,16 +3976,16 @@
           <t>5 days</t>
         </is>
       </c>
-      <c r="H64" s="38" t="inlineStr">
+      <c r="H64" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I64" s="34" t="inlineStr"/>
+      <c r="I64" s="44" t="inlineStr"/>
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="B65" s="14" t="inlineStr"/>
-      <c r="C65" s="31" t="inlineStr">
+      <c r="C65" s="41" t="inlineStr">
         <is>
           <t>GitHub Actions CI pipeline (type-check + lint + Vitest + Playwright + SSH deploy on merge)</t>
         </is>
@@ -3577,16 +4010,16 @@
           <t>2 days</t>
         </is>
       </c>
-      <c r="H65" s="38" t="inlineStr">
+      <c r="H65" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I65" s="34" t="inlineStr"/>
+      <c r="I65" s="44" t="inlineStr"/>
     </row>
     <row r="66" ht="20" customHeight="1">
       <c r="B66" s="14" t="inlineStr"/>
-      <c r="C66" s="31" t="inlineStr">
+      <c r="C66" s="41" t="inlineStr">
         <is>
           <t>Production environment setup (Docker Compose + Nginx + self-hosted Postgres + Redis on client's server)</t>
         </is>
@@ -3611,16 +4044,16 @@
           <t>1 day</t>
         </is>
       </c>
-      <c r="H66" s="32" t="inlineStr">
+      <c r="H66" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="I66" s="34" t="inlineStr"/>
+      <c r="I66" s="44" t="inlineStr"/>
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="B67" s="14" t="inlineStr"/>
-      <c r="C67" s="31" t="inlineStr">
+      <c r="C67" s="41" t="inlineStr">
         <is>
           <t>Custom domain + SSL (Let's Encrypt via Certbot + Nginx) + env var management</t>
         </is>
@@ -3645,12 +4078,12 @@
           <t>1 day</t>
         </is>
       </c>
-      <c r="H67" s="38" t="inlineStr">
+      <c r="H67" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I67" s="33" t="inlineStr">
+      <c r="I67" s="43" t="inlineStr">
         <is>
           <t>Nginx handles SSL termination</t>
         </is>
@@ -3658,7 +4091,7 @@
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="B68" s="14" t="inlineStr"/>
-      <c r="C68" s="31" t="inlineStr">
+      <c r="C68" s="41" t="inlineStr">
         <is>
           <t>DB migration strategy (Drizzle migrate on deploy, zero-downtime)</t>
         </is>
@@ -3683,12 +4116,12 @@
           <t>1 day</t>
         </is>
       </c>
-      <c r="H68" s="38" t="inlineStr">
+      <c r="H68" s="48" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I68" s="34" t="inlineStr"/>
+      <c r="I68" s="44" t="inlineStr"/>
     </row>
     <row r="69" ht="20" customHeight="1">
       <c r="B69" s="8" t="inlineStr">
@@ -3696,7 +4129,7 @@
           <t>Phase 7 Total</t>
         </is>
       </c>
-      <c r="C69" s="35" t="inlineStr"/>
+      <c r="C69" s="45" t="inlineStr"/>
       <c r="D69" s="8" t="inlineStr">
         <is>
           <t>6.5 days</t>
@@ -3717,8 +4150,8 @@
           <t>15 days</t>
         </is>
       </c>
-      <c r="H69" s="36" t="inlineStr"/>
-      <c r="I69" s="37" t="inlineStr"/>
+      <c r="H69" s="46" t="inlineStr"/>
+      <c r="I69" s="47" t="inlineStr"/>
     </row>
     <row r="70" ht="26" customHeight="1">
       <c r="B70" s="17" t="inlineStr">
@@ -3726,7 +4159,7 @@
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C70" s="40" t="inlineStr">
+      <c r="C70" s="50" t="inlineStr">
         <is>
           <t>All Phases (1–7)  ·  556 hrs  ·  $20/hr</t>
         </is>
@@ -3751,8 +4184,8 @@
           <t>163 days</t>
         </is>
       </c>
-      <c r="H70" s="36" t="inlineStr"/>
-      <c r="I70" s="33" t="inlineStr">
+      <c r="H70" s="46" t="inlineStr"/>
+      <c r="I70" s="43" t="inlineStr">
         <is>
           <t>Wall-clock: ~3–4 weeks with parallelism</t>
         </is>
@@ -3794,60 +4227,60 @@
   </cols>
   <sheetData>
     <row r="1" ht="50" customHeight="1">
-      <c r="B1" s="28" t="inlineStr">
+      <c r="B1" s="38" t="inlineStr">
         <is>
           <t>DecisionOS — 3–4 Week Delivery Plan</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="B2" s="29" t="inlineStr">
+      <c r="B2" s="39" t="inlineStr">
         <is>
           <t>5 parallel Claude Code SDD agent streams · 69.5 AI days ÷ ~4.5 avg streams ≈ 15 effective days + buffer = 3–4 weeks · Total dev cost: $11,120 @ $20/hr</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="51" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="C4" s="42" t="inlineStr">
+      <c r="C4" s="52" t="inlineStr">
         <is>
           <t>Stream A</t>
         </is>
       </c>
-      <c r="D4" s="43" t="inlineStr">
+      <c r="D4" s="53" t="inlineStr">
         <is>
           <t>Stream B</t>
         </is>
       </c>
-      <c r="E4" s="44" t="inlineStr">
+      <c r="E4" s="54" t="inlineStr">
         <is>
           <t>Stream C</t>
         </is>
       </c>
-      <c r="F4" s="45" t="inlineStr">
+      <c r="F4" s="55" t="inlineStr">
         <is>
           <t>Stream D</t>
         </is>
       </c>
-      <c r="G4" s="46" t="inlineStr">
+      <c r="G4" s="56" t="inlineStr">
         <is>
           <t>Stream E</t>
         </is>
       </c>
     </row>
     <row r="5" ht="95" customHeight="1">
-      <c r="B5" s="47" t="inlineStr">
+      <c r="B5" s="57" t="inlineStr">
         <is>
           <t>Week 1
 Foundation
 $1,760</t>
         </is>
       </c>
-      <c r="C5" s="48" t="inlineStr">
+      <c r="C5" s="58" t="inlineStr">
         <is>
           <t>Phase 1: PostgreSQL schema
 (all 7 table groups)
@@ -3855,21 +4288,21 @@
 + self-hosted Postgres</t>
         </is>
       </c>
-      <c r="D5" s="49" t="inlineStr">
+      <c r="D5" s="59" t="inlineStr">
         <is>
           <t>Phase 1: Auth.js v5
 + bcrypt + JWT
 + httpOnly cookie</t>
         </is>
       </c>
-      <c r="E5" s="48" t="inlineStr">
+      <c r="E5" s="58" t="inlineStr">
         <is>
           <t>Phase 1: Schema-per-tenant
 middleware
 + Zod API scaffold</t>
         </is>
       </c>
-      <c r="F5" s="49" t="inlineStr">
+      <c r="F5" s="59" t="inlineStr">
         <is>
           <t>Phase 7: CI/CD pipeline
 (GitHub Actions,
@@ -3877,7 +4310,7 @@
 Nginx + Let's Encrypt)</t>
         </is>
       </c>
-      <c r="G5" s="48" t="inlineStr">
+      <c r="G5" s="58" t="inlineStr">
         <is>
           <t>Phase 2: File upload
 + local disk storage
@@ -3886,14 +4319,14 @@
       </c>
     </row>
     <row r="6" ht="95" customHeight="1">
-      <c r="B6" s="50" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>Week 2
 Core AI
 $2,880</t>
         </is>
       </c>
-      <c r="C6" s="49" t="inlineStr">
+      <c r="C6" s="59" t="inlineStr">
         <is>
           <t>Phase 4: pgvector
 + embedding pipeline
@@ -3901,28 +4334,28 @@
 LLM adapters</t>
         </is>
       </c>
-      <c r="D6" s="48" t="inlineStr">
+      <c r="D6" s="58" t="inlineStr">
         <is>
           <t>Phase 4: RAG retrieval
 + SQL generation
 + chat sessions API</t>
         </is>
       </c>
-      <c r="E6" s="49" t="inlineStr">
+      <c r="E6" s="59" t="inlineStr">
         <is>
           <t>Phase 3: Zoho CRM
 OAuth + data sync
 + encrypted credentials</t>
         </is>
       </c>
-      <c r="F6" s="48" t="inlineStr">
+      <c r="F6" s="58" t="inlineStr">
         <is>
           <t>Phase 2: CSV/Excel
 parser + schema
 inference + dynamic DDL</t>
         </is>
       </c>
-      <c r="G6" s="49" t="inlineStr">
+      <c r="G6" s="59" t="inlineStr">
         <is>
           <t>Phase 5: TanStack hooks
 for Phase 1 endpoints
@@ -3931,42 +4364,42 @@
       </c>
     </row>
     <row r="7" ht="95" customHeight="1">
-      <c r="B7" s="51" t="inlineStr">
+      <c r="B7" s="61" t="inlineStr">
         <is>
           <t>Week 3
 Full AI + Admin
 $4,000</t>
         </is>
       </c>
-      <c r="C7" s="48" t="inlineStr">
+      <c r="C7" s="58" t="inlineStr">
         <is>
           <t>Phase 4: 7-agent
 orchestration pipeline
 + SSE streaming</t>
         </is>
       </c>
-      <c r="D7" s="49" t="inlineStr">
+      <c r="D7" s="59" t="inlineStr">
         <is>
           <t>Phase 4: LLM connect
 wizard + usage logging
 + AI exec summary</t>
         </is>
       </c>
-      <c r="E7" s="48" t="inlineStr">
+      <c r="E7" s="58" t="inlineStr">
         <is>
           <t>Phase 5: Subscription
 enforcement + Tenant
 Admin + Platform Admin</t>
         </is>
       </c>
-      <c r="F7" s="49" t="inlineStr">
+      <c r="F7" s="59" t="inlineStr">
         <is>
           <t>Phase 3: Custom ERP
 connector + pg-boss
 sync scheduler</t>
         </is>
       </c>
-      <c r="G7" s="48" t="inlineStr">
+      <c r="G7" s="58" t="inlineStr">
         <is>
           <t>Phase 6: Redis rate
 limiting + Sentry
@@ -3975,34 +4408,34 @@
       </c>
     </row>
     <row r="8" ht="95" customHeight="1">
-      <c r="B8" s="52" t="inlineStr">
+      <c r="B8" s="62" t="inlineStr">
         <is>
           <t>Week 4
 QA + Deploy
 $2,480</t>
         </is>
       </c>
-      <c r="C8" s="49" t="inlineStr">
+      <c r="C8" s="59" t="inlineStr">
         <is>
           <t>Phase 4: Insight +
 Recommendation
 auto-generation (cron)</t>
         </is>
       </c>
-      <c r="D8" s="48" t="inlineStr">
+      <c r="D8" s="58" t="inlineStr">
         <is>
           <t>Phase 5: Real charts
 + notification system
 + workflow persistence</t>
         </is>
       </c>
-      <c r="E8" s="49" t="inlineStr">
+      <c r="E8" s="59" t="inlineStr">
         <is>
           <t>Phase 7: Vitest unit
 + integration tests</t>
         </is>
       </c>
-      <c r="F8" s="48" t="inlineStr">
+      <c r="F8" s="58" t="inlineStr">
         <is>
           <t>Phase 7: Playwright E2E
 + production deploy
@@ -4010,7 +4443,7 @@
 + client server)</t>
         </is>
       </c>
-      <c r="G8" s="49" t="inlineStr">
+      <c r="G8" s="59" t="inlineStr">
         <is>
           <t>Phase 6: Security audit
 + data isolation
@@ -4053,7 +4486,7 @@
           <t>Foundation Live</t>
         </is>
       </c>
-      <c r="D12" s="31" t="inlineStr">
+      <c r="D12" s="41" t="inlineStr">
         <is>
           <t>Real login + self-hosted Postgres live + file upload to local disk + CI/CD running</t>
         </is>
@@ -4070,7 +4503,7 @@
           <t>Core Value Prop Working</t>
         </is>
       </c>
-      <c r="D13" s="31" t="inlineStr">
+      <c r="D13" s="41" t="inlineStr">
         <is>
           <t>Upload CSV → Ask AI answers · Zoho CRM syncing · Dashboard KPIs live · Chat history persisted</t>
         </is>
@@ -4087,7 +4520,7 @@
           <t>Full AI + All Connectors</t>
         </is>
       </c>
-      <c r="D14" s="31" t="inlineStr">
+      <c r="D14" s="41" t="inlineStr">
         <is>
           <t>7-agent AI chain + SSE streaming · All connectors live · Admin consoles · Rate limiting</t>
         </is>
@@ -4104,7 +4537,7 @@
           <t>Production Deployed</t>
         </is>
       </c>
-      <c r="D15" s="31" t="inlineStr">
+      <c r="D15" s="41" t="inlineStr">
         <is>
           <t>Production URL + custom domain + SSL · Playwright E2E passing · Security audit clean</t>
         </is>
@@ -4144,14 +4577,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="50" customHeight="1">
-      <c r="B1" s="28" t="inlineStr">
+      <c r="B1" s="38" t="inlineStr">
         <is>
           <t>DecisionOS — Subscription Plans</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="B2" s="29" t="inlineStr">
+      <c r="B2" s="39" t="inlineStr">
         <is>
           <t>Tenants bring their own LLM API keys and pay the LLM provider directly. Plans gate integrations + platform limits.</t>
         </is>
@@ -4163,7 +4596,7 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="C4" s="53" t="inlineStr">
+      <c r="C4" s="63" t="inlineStr">
         <is>
           <t>Trial</t>
         </is>
@@ -4173,12 +4606,12 @@
           <t>Starter</t>
         </is>
       </c>
-      <c r="E4" s="54" t="inlineStr">
+      <c r="E4" s="64" t="inlineStr">
         <is>
           <t>Professional</t>
         </is>
       </c>
-      <c r="F4" s="55" t="inlineStr">
+      <c r="F4" s="65" t="inlineStr">
         <is>
           <t>Enterprise</t>
         </is>
@@ -4212,7 +4645,7 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="56" t="inlineStr">
+      <c r="B6" s="66" t="inlineStr">
         <is>
           <t>Users</t>
         </is>
@@ -4266,7 +4699,7 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="B8" s="56" t="inlineStr">
+      <c r="B8" s="66" t="inlineStr">
         <is>
           <t>AI Query Cap</t>
         </is>
@@ -4320,12 +4753,12 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="56" t="inlineStr">
+      <c r="B10" s="66" t="inlineStr">
         <is>
           <t>OpenAI GPT-4o</t>
         </is>
       </c>
-      <c r="C10" s="57" t="inlineStr">
+      <c r="C10" s="67" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -4352,7 +4785,7 @@
           <t>Anthropic Claude Haiku</t>
         </is>
       </c>
-      <c r="C11" s="57" t="inlineStr">
+      <c r="C11" s="67" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -4374,17 +4807,17 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="56" t="inlineStr">
+      <c r="B12" s="66" t="inlineStr">
         <is>
           <t>Anthropic Claude Sonnet</t>
         </is>
       </c>
-      <c r="C12" s="57" t="inlineStr">
+      <c r="C12" s="67" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="D12" s="57" t="inlineStr">
+      <c r="D12" s="67" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -4406,12 +4839,12 @@
           <t>Google Gemini Pro</t>
         </is>
       </c>
-      <c r="C13" s="57" t="inlineStr">
+      <c r="C13" s="67" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="D13" s="57" t="inlineStr">
+      <c r="D13" s="67" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -4428,22 +4861,22 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="56" t="inlineStr">
+      <c r="B14" s="66" t="inlineStr">
         <is>
           <t>Ollama (self-hosted)</t>
         </is>
       </c>
-      <c r="C14" s="57" t="inlineStr">
+      <c r="C14" s="67" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="D14" s="57" t="inlineStr">
+      <c r="D14" s="67" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E14" s="57" t="inlineStr">
+      <c r="E14" s="67" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -4460,17 +4893,17 @@
           <t>Custom model endpoints</t>
         </is>
       </c>
-      <c r="C15" s="57" t="inlineStr">
+      <c r="C15" s="67" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="D15" s="57" t="inlineStr">
+      <c r="D15" s="67" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="E15" s="57" t="inlineStr">
+      <c r="E15" s="67" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
@@ -4482,7 +4915,7 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="56" t="inlineStr">
+      <c r="B16" s="66" t="inlineStr">
         <is>
           <t>LLM Usage Dashboard</t>
         </is>
@@ -4536,7 +4969,7 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="56" t="inlineStr">
+      <c r="B18" s="66" t="inlineStr">
         <is>
           <t>Custom ERP connector</t>
         </is>
@@ -4590,7 +5023,7 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="B20" s="56" t="inlineStr">
+      <c r="B20" s="66" t="inlineStr">
         <is>
           <t>AI Insights + Recs</t>
         </is>
@@ -4644,7 +5077,7 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="56" t="inlineStr">
+      <c r="B22" s="66" t="inlineStr">
         <is>
           <t>Support</t>
         </is>
@@ -4705,7 +5138,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="50" customHeight="1">
-      <c r="B1" s="28" t="inlineStr">
+      <c r="B1" s="38" t="inlineStr">
         <is>
           <t>Open Items &amp; Client Dependencies</t>
         </is>
@@ -4734,19 +5167,19 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="B4" s="58" t="inlineStr">
+      <c r="B4" s="68" t="inlineStr">
         <is>
           <t>✅ ANSWERED</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
-      <c r="B5" s="59" t="inlineStr">
+      <c r="B5" s="69" t="inlineStr">
         <is>
           <t>LLM API key model</t>
         </is>
       </c>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="41" t="inlineStr">
         <is>
           <t>Tenants bring their own keys and pay the LLM provider directly.</t>
         </is>
@@ -4756,19 +5189,19 @@
           <t>Confirmed</t>
         </is>
       </c>
-      <c r="E5" s="60" t="inlineStr">
+      <c r="E5" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
-      <c r="B6" s="59" t="inlineStr">
+      <c r="B6" s="69" t="inlineStr">
         <is>
           <t>Delivery target</t>
         </is>
       </c>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="C6" s="41" t="inlineStr">
         <is>
           <t>3–4 weeks via 5 parallel Claude Code SDD agent streams.</t>
         </is>
@@ -4778,19 +5211,19 @@
           <t>Confirmed</t>
         </is>
       </c>
-      <c r="E6" s="60" t="inlineStr">
+      <c r="E6" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
-      <c r="B7" s="59" t="inlineStr">
+      <c r="B7" s="69" t="inlineStr">
         <is>
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="C7" s="31" t="inlineStr">
+      <c r="C7" s="41" t="inlineStr">
         <is>
           <t>Client's on-premise server. Self-hosted Postgres + Redis + local disk. GitHub + Sentry only external services.</t>
         </is>
@@ -4800,19 +5233,19 @@
           <t>Confirmed</t>
         </is>
       </c>
-      <c r="E7" s="60" t="inlineStr">
+      <c r="E7" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
-      <c r="B8" s="59" t="inlineStr">
+      <c r="B8" s="69" t="inlineStr">
         <is>
           <t>Development rate</t>
         </is>
       </c>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="C8" s="41" t="inlineStr">
         <is>
           <t>$20/hr × 8 hrs/day. Total: 69.5 days × $160/day = $11,120.</t>
         </is>
@@ -4822,26 +5255,26 @@
           <t>Confirmed</t>
         </is>
       </c>
-      <c r="E8" s="60" t="inlineStr">
+      <c r="E8" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="61" t="inlineStr">
+      <c r="B9" s="71" t="inlineStr">
         <is>
           <t>⚠️ PENDING — CLIENT ACTION REQUIRED</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
-      <c r="B10" s="62" t="inlineStr">
+      <c r="B10" s="72" t="inlineStr">
         <is>
           <t>Custom ERP API documentation</t>
         </is>
       </c>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="C10" s="41" t="inlineStr">
         <is>
           <t>Share base URL, auth type, and key endpoint schemas. Without docs, ERP connector cannot be scoped.</t>
         </is>
@@ -4851,19 +5284,19 @@
           <t>Client</t>
         </is>
       </c>
-      <c r="E10" s="63" t="inlineStr">
+      <c r="E10" s="73" t="inlineStr">
         <is>
           <t>HIGH — ERP connector deferred to sprint 2</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
-      <c r="B11" s="62" t="inlineStr">
+      <c r="B11" s="72" t="inlineStr">
         <is>
           <t>Zoho app registration</t>
         </is>
       </c>
-      <c r="C11" s="31" t="inlineStr">
+      <c r="C11" s="41" t="inlineStr">
         <is>
           <t>Register a Server-based App in Zoho Developer Console (free). Share client_id + client_secret by Day 3.</t>
         </is>
@@ -4873,19 +5306,19 @@
           <t>Client</t>
         </is>
       </c>
-      <c r="E11" s="62" t="inlineStr">
+      <c r="E11" s="72" t="inlineStr">
         <is>
           <t>MEDIUM — Zoho sync delayed</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
-      <c r="B12" s="62" t="inlineStr">
+      <c r="B12" s="72" t="inlineStr">
         <is>
           <t>Tenant LLM API keys for testing</t>
         </is>
       </c>
-      <c r="C12" s="31" t="inlineStr">
+      <c r="C12" s="41" t="inlineStr">
         <is>
           <t>Share an OpenAI or Anthropic API key for end-to-end testing of Ask AI. Required by start of Week 2.</t>
         </is>
@@ -4895,19 +5328,19 @@
           <t>Client</t>
         </is>
       </c>
-      <c r="E12" s="62" t="inlineStr">
+      <c r="E12" s="72" t="inlineStr">
         <is>
           <t>MEDIUM — AI testing blocked</t>
         </is>
       </c>
     </row>
     <row r="13" ht="38" customHeight="1">
-      <c r="B13" s="62" t="inlineStr">
+      <c r="B13" s="72" t="inlineStr">
         <is>
           <t>DNS / custom domain</t>
         </is>
       </c>
-      <c r="C13" s="31" t="inlineStr">
+      <c r="C13" s="41" t="inlineStr">
         <is>
           <t>Point your domain's A record to the server's IP address. We provide the IP once server is set up.</t>
         </is>
@@ -4917,26 +5350,26 @@
           <t>Client</t>
         </is>
       </c>
-      <c r="E13" s="60" t="inlineStr">
+      <c r="E13" s="70" t="inlineStr">
         <is>
           <t>LOW — Custom domain delayed</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="64" t="inlineStr">
+      <c r="B14" s="74" t="inlineStr">
         <is>
           <t>❓ OPEN QUESTIONS</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
-      <c r="B15" s="62" t="inlineStr">
+      <c r="B15" s="72" t="inlineStr">
         <is>
           <t>Number of launch tenants</t>
         </is>
       </c>
-      <c r="C15" s="31" t="inlineStr">
+      <c r="C15" s="41" t="inlineStr">
         <is>
           <t>How many tenant organisations at go-live? Informs connection pool sizing on self-hosted Postgres.</t>
         </is>
@@ -4946,19 +5379,19 @@
           <t>Client</t>
         </is>
       </c>
-      <c r="E15" s="60" t="inlineStr">
+      <c r="E15" s="70" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
-      <c r="B16" s="62" t="inlineStr">
+      <c r="B16" s="72" t="inlineStr">
         <is>
           <t>Zoho plan tier</t>
         </is>
       </c>
-      <c r="C16" s="31" t="inlineStr">
+      <c r="C16" s="41" t="inlineStr">
         <is>
           <t>Free = 100 API req/min; Professional+ = higher limits. Affects delta sync frequency.</t>
         </is>
@@ -4968,19 +5401,19 @@
           <t>Client</t>
         </is>
       </c>
-      <c r="E16" s="60" t="inlineStr">
+      <c r="E16" s="70" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="17" ht="38" customHeight="1">
-      <c r="B17" s="62" t="inlineStr">
+      <c r="B17" s="72" t="inlineStr">
         <is>
           <t>Post-launch: Stripe billing</t>
         </is>
       </c>
-      <c r="C17" s="31" t="inlineStr">
+      <c r="C17" s="41" t="inlineStr">
         <is>
           <t>Self-serve plan upgrade/downgrade via Stripe (~3 days). Confirm if needed in sprint 2.</t>
         </is>
@@ -4990,7 +5423,7 @@
           <t>Client</t>
         </is>
       </c>
-      <c r="E17" s="60" t="inlineStr">
+      <c r="E17" s="70" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>

</xml_diff>